<commit_message>
Correct ID input variable
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-FRA.xlsx
+++ b/baseline/data_processing_elements-FRA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\FRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001A0AB1-13F7-4D7F-8E42-7C06865F247F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8B48E6-3774-4CAB-AA95-70A02686DF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CCDECE63-0FFC-4822-923F-34FACAF497E3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1896" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="670">
   <si>
     <t>index</t>
   </si>
@@ -3026,21 +3026,24 @@
         <v>27</v>
       </c>
       <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s">
         <v>28</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>29</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>31</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>33</v>
       </c>
       <c r="U2" t="s">

</xml_diff>

<commit_message>
correct harmo error during meeting
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-FRA.xlsx
+++ b/baseline/data_processing_elements-FRA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\FRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8B48E6-3774-4CAB-AA95-70A02686DF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E32CC9-4B21-4B0E-B4D4-12415C205242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CCDECE63-0FFC-4822-923F-34FACAF497E3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="671">
   <si>
     <t>index</t>
   </si>
@@ -1700,6 +1700,781 @@
 med1atc1;
 ...;
 med9atc1</t>
+  </si>
+  <si>
+    <t>dis_msk_ever</t>
+  </si>
+  <si>
+    <t>Musculoskeletal diseases ever</t>
+  </si>
+  <si>
+    <t>Musculoskeletal diseases ever (osteoporosis, arthrosis, rheumatic disorder, osteoarthritis or rheumatism, rheumatoid arthritis, osteoarthritis, other arthritis, rheumatoid arthritis)</t>
+  </si>
+  <si>
+    <t>A "No" response can be assigned if the input variables were collected in Yes/No format. 
+If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
+  </si>
+  <si>
+    <t>osteoarthrosis1;
+osteoporosis1;
+sciatica1;
+rheumatoidarthritis1</t>
+  </si>
+  <si>
+    <t>Osteoarthrosis;
+Osteoporosis;
+Sciatica (lumbar disc herniation);
+Rheumatoid arthritis</t>
+  </si>
+  <si>
+    <t>HAM_LSI;HAM_LSI;HAM_LSI;HAM_LSI;HAM_LSI</t>
+  </si>
+  <si>
+    <t>Osteoarthrosis. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of osteoarthrosis? Response options: no, yes: previously, yes: currently;
+Osteoporosiss. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of osteoporosis? Response options: no, yes: previously, yes: currently;
+Sciatica (lumbar disc herniation). Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of sciatica (lumbar disc herniation)? Response options: no, yes: previously, yes: currently ;
+Fibromyalgia. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of fibromyalgia? Response options: no, yes: previously, yes: currently ;
+Rheumatoid arthritis. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of rheumatoid arthritis? Response options: no, yes: previously, yes: currently</t>
+  </si>
+  <si>
+    <t>Cohort profile: DOI: 10.1093/gerona/glaa193
+;Cohort profile: DOI: 10.1093/gerona/glaa193
+;Cohort profile: DOI: 10.1093/gerona/glaa193
+;Cohort profile: DOI: 10.1093/gerona/glaa193
+;Cohort profile: DOI: 10.1093/gerona/glaa193</t>
+  </si>
+  <si>
+    <t>case_when(
+osteoarthrosis1 %in% c(2, 3) | osteoporosis1 %in% c(2, 3) | sciatica1 %in% c(2, 3) | rheumatoidarthritis1 %in% c(2, 3) ~ 1L;
+osteoarthrosis1 == 1 &amp; osteoporosis1 == 1 &amp; sciatica1 == 1 &amp; rheumatoidarthritis1 == 1 ~ 0L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>dis_diabetes</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
+    <t>Diabetes (including gestational diabetes and other types of diabetes but excluding impaired fasting glucose and impaired glucose tolerance)</t>
+  </si>
+  <si>
+    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
+If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned. 
+Add a harmonization comment about any study-specific wording for collecting information about diabetes (e.g., only Type 2 diabetes, excluding gestational diabetes).</t>
+  </si>
+  <si>
+    <t>diabetes1</t>
+  </si>
+  <si>
+    <t>Type 2 diabetes</t>
+  </si>
+  <si>
+    <t>Type 2 diabetes. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of type 2 diabetes? Response options: no, yes: previously, yes: currently.</t>
+  </si>
+  <si>
+    <t>1 = no 
+2 = yes, previously 
+3 = yes, currently</t>
+  </si>
+  <si>
+    <t>The study only ask about type 2 diabetes.</t>
+  </si>
+  <si>
+    <t>dis_diabetes_type</t>
+  </si>
+  <si>
+    <t>Diabetes type</t>
+  </si>
+  <si>
+    <t>Add a harmonization comment about any study-specific wording for collecting information about diabetes (e.g., only Type 2 diabetes collected).</t>
+  </si>
+  <si>
+    <t>1 Type 1 
+2 Type 2 
+3 Other</t>
+  </si>
+  <si>
+    <t>dis_cancer_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever</t>
+  </si>
+  <si>
+    <t>When studies do not have an "other cancer" category, a "No" cannot be generated. In this situation only 1 and NA would be present.
+Add a harmonization comment about any decisions made for harmonization.
+"Presumed no" can be specified only if a general cancer disease option is present in a select all that apply question where at least another option is selected but not this one.</t>
+  </si>
+  <si>
+    <t>malignanttumor1</t>
+  </si>
+  <si>
+    <t>Malignant tumor (cancer)</t>
+  </si>
+  <si>
+    <t>Malignant tumor (cancer). Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of malignant tumor? Response options: no, yes: previously, yes: currently</t>
+  </si>
+  <si>
+    <t>dis_cancer_bladder_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Bladder</t>
+  </si>
+  <si>
+    <t>The "No" response can be attributed only in 2 situations:
+- There is a parent variable about having any cancer, collected in Yes/No format.
+- The input variables were collected in Yes/No format for this specific cancer type
+If the input variables do not have a "No" response but are part of select all that apply section where at least another cancer type is selected, then a "Presumed no" can be assigned.</t>
+  </si>
+  <si>
+    <t>case_when(
+malignanttumor1 == 1 ~ 0L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>dis_cancer_breast_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Breast</t>
+  </si>
+  <si>
+    <t>dis_cancer_cervix_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Cervix</t>
+  </si>
+  <si>
+    <t>dis_cancer_colorectal_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Colon-Rectum</t>
+  </si>
+  <si>
+    <t>dis_cancer_kidney_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Kidney</t>
+  </si>
+  <si>
+    <t>dis_cancer_throat_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Throat/Larynx-Pharynx</t>
+  </si>
+  <si>
+    <t>dis_cancer_leukaemia_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Leukaemia</t>
+  </si>
+  <si>
+    <t>dis_cancer_lung_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Lung</t>
+  </si>
+  <si>
+    <t>dis_cancer_lymphoma_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Lymphoma</t>
+  </si>
+  <si>
+    <t>dis_cancer_prostate_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Prostate</t>
+  </si>
+  <si>
+    <t>dis_cancer_skin_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Skin</t>
+  </si>
+  <si>
+    <t>dis_cancer_stomach_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Stomach</t>
+  </si>
+  <si>
+    <t>dis_cancer_testicle_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Testicle</t>
+  </si>
+  <si>
+    <t>dis_cancer_uterus_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Uterus</t>
+  </si>
+  <si>
+    <t>dis_cancer_brain_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Brain</t>
+  </si>
+  <si>
+    <t>dis_cancer_liver_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Liver</t>
+  </si>
+  <si>
+    <t>dis_cancer_ovary_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Ovary</t>
+  </si>
+  <si>
+    <t>dis_cancer_pancreas_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Pancreas</t>
+  </si>
+  <si>
+    <t>dis_cancer_thyroid_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Thyroid</t>
+  </si>
+  <si>
+    <t>dis_hypercholesteromia_ever</t>
+  </si>
+  <si>
+    <t>Diagnosed hypercholesteromia</t>
+  </si>
+  <si>
+    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
+If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
+  </si>
+  <si>
+    <t>highcholesterol1</t>
+  </si>
+  <si>
+    <t>High cholesterol</t>
+  </si>
+  <si>
+    <t>High cholesterol. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of high cholesterol? Response options: no, yes: previously, yes: currently.</t>
+  </si>
+  <si>
+    <t>dis_depression</t>
+  </si>
+  <si>
+    <t>Depression</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant has depression or not</t>
+  </si>
+  <si>
+    <t>Accept self-reported condition but with a note. 
+A "No" response can be assigned if the input variables were collected in Yes/No format.
+If the input variable do not have a "No" response but is part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
+  </si>
+  <si>
+    <t>depression1</t>
+  </si>
+  <si>
+    <t>depression</t>
+  </si>
+  <si>
+    <t>HAM_Depression</t>
+  </si>
+  <si>
+    <t>Depression. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of depression? Response options: no, yes: previously, yes: currently.</t>
+  </si>
+  <si>
+    <t>dis_alzheimers_dementia</t>
+  </si>
+  <si>
+    <t>Alzheimers/Dementia</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant has Alzheimers/Dementia</t>
+  </si>
+  <si>
+    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
+If the input variable do not have a "No" response but is part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 Has not been diagnosed with Alzheimers or other dementia 
+1 Has been diagnosed with Alzheimers or other dementia 
+2 Has presumably not been diagnosed with Alzheimers or other dementia 
+</t>
+  </si>
+  <si>
+    <t>alzheimer1</t>
+  </si>
+  <si>
+    <t>Alzheimer or other dementia</t>
+  </si>
+  <si>
+    <t>HAM_Alzheimers</t>
+  </si>
+  <si>
+    <t>Alzheimer or other dementia. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of Alzheimer or other dementia? Response options: no, yes: previously, yes: currently.</t>
+  </si>
+  <si>
+    <t>med_lipid_lowering_cur</t>
+  </si>
+  <si>
+    <t>Current use of lipid lowering medication</t>
+  </si>
+  <si>
+    <t>Only include if lipid lowering medication is currently being taken. A "No" response is possible only if a Yes/No question is collected.
+If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
+  </si>
+  <si>
+    <t>med1atc1;
+med2atc1;
+med3atc1;
+med4atc1;
+med5atc1;
+med6atc1;
+med7atc1;
+med8atc1;
+med9atc1</t>
+  </si>
+  <si>
+    <t>Medication 1 to 5 atc code</t>
+  </si>
+  <si>
+    <t>HAM_MedUse</t>
+  </si>
+  <si>
+    <t>ATC code (Anatomical Therapeutic Chemical classification) of the medication used. Self-reported. Participants were asked to fill in a form names of medicines that they used. The full ATC code (A10BH01 etc). If the ATC code was not found, medicine was coded as follows: 
+X01= anti-hypertensive drug
+X02= diabetes drug
+X03= analgesic (painkiller)
+X04= cholesterol medicine
+X05= hormone replacement therapy
+X06= cortisone
+X07= vitamin 
+X08= nature cure/alternative remedy
+X10= something else/unspecified
+X11= antidepressant
+X12= allergy medicine
+X13= cortisone salve</t>
+  </si>
+  <si>
+    <t>ATC code (Anatomical Therapeutic Chemical classification)
+or if ATC code missing: 
+X01= anti-hypertensive drug
+X02= diabetes drug
+X03= analgesic (painkiller)
+X04= cholesterol medicine
+X05= hormone replacement therapy
+X06= cortisone
+X07= vitamin 
+X08= nature cure/alternative remedy
+X10= something else/unspecified
+X11= antidepressant
+X12= allergy medicine
+X13= cortisone salve</t>
+  </si>
+  <si>
+    <t>Derived from list of medication taken by the participant.</t>
+  </si>
+  <si>
+    <t>case_when(
+med1atc1 == "X04" ~ 1L;
+med2atc1 == "X04" ~ 1L;
+med3atc1 == "X04" ~ 1L;
+med4atc1 == "X04" ~ 1L;
+med5atc1 == "X04" ~ 1L;
+med6atc1 == "X04" ~ 1L;
+med7atc1 == "X04" ~ 1L;
+med8atc1 == "X04" ~ 1L;
+med9atc1 == "X04" ~ 1L;
+grepl("^C10", med1atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med2atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med3atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med4atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med5atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med6atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med7atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med8atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C10", med9atc1, ignore.case = TRUE) ~ 1L;
+!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>med_blood_pressure_cur</t>
+  </si>
+  <si>
+    <t>Current use of medication to manage blood pressure</t>
+  </si>
+  <si>
+    <t>Only include if medication for hypertension or high blood pressure is currently being taken. A "No" response is possible only if a Yes/No question is collected.
+The question must be separated from a hypertension or hbp diagnosis question.
+If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
+  </si>
+  <si>
+    <t>case_when(
+med1atc1 == "X01" ~ 1L;
+med2atc1 == "X01" ~ 1L;
+med3atc1 == "X01" ~ 1L;
+med4atc1 == "X01" ~ 1L;
+med5atc1 == "X01" ~ 1L;
+med6atc1 == "X01" ~ 1L;
+med7atc1 == "X01" ~ 1L;
+med8atc1 == "X01" ~ 1L;
+med9atc1 == "X01" ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med1atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med2atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med3atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med4atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med5atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med6atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med7atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med8atc1, ignore.case = TRUE) ~ 1L;
+grepl("^C02|^C03|^C07|^C08|^C09", med9atc1, ignore.case = TRUE) ~ 1L;
+!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>med_diabetes_cur</t>
+  </si>
+  <si>
+    <t>Current use of medication for diabetes</t>
+  </si>
+  <si>
+    <t>If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
+  </si>
+  <si>
+    <t>case_when(
+med1atc1 == "X02" ~ 1L;
+med2atc1 == "X02" ~ 1L;
+med3atc1 == "X02" ~ 1L;
+med4atc1 == "X02" ~ 1L;
+med5atc1 == "X02" ~ 1L;
+med6atc1 == "X02" ~ 1L;
+med7atc1 == "X02" ~ 1L;
+med8atc1 == "X02" ~ 1L;
+med9atc1 == "X02" ~ 1L;
+grepl("^A10", med1atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med2atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med3atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med4atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med5atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med6atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med7atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med8atc1, ignore.case = TRUE) ~ 1L;
+grepl("^A10", med9atc1, ignore.case = TRUE) ~ 1L;
+!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>psy_dep_cesd20</t>
+  </si>
+  <si>
+    <t>CES-D (20 items) score</t>
+  </si>
+  <si>
+    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-60</t>
+  </si>
+  <si>
+    <t>psy_dep_cesd10</t>
+  </si>
+  <si>
+    <t>CES-D (10 items) score</t>
+  </si>
+  <si>
+    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-30</t>
+  </si>
+  <si>
+    <t>psy_dep_malaise</t>
+  </si>
+  <si>
+    <t>Malaise inventory (9 items) score</t>
+  </si>
+  <si>
+    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-24</t>
+  </si>
+  <si>
+    <t>psy_dep_kessler</t>
+  </si>
+  <si>
+    <t>Kessler psychological distress score</t>
+  </si>
+  <si>
+    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 10-50</t>
+  </si>
+  <si>
+    <t>psy_dep_phq9</t>
+  </si>
+  <si>
+    <t>PHQ-9 score</t>
+  </si>
+  <si>
+    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-27</t>
+  </si>
+  <si>
+    <t>psy_mci_mmse_score</t>
+  </si>
+  <si>
+    <t>MMSE score</t>
+  </si>
+  <si>
+    <t>mci1</t>
+  </si>
+  <si>
+    <t>Mild cognitive impairment</t>
+  </si>
+  <si>
+    <t>HAM_MildCI</t>
+  </si>
+  <si>
+    <t>Mild cognitive impairment was assessed during a clinical study visit with the Mini-Mental State Examination (MMSE) including items to assess cognitive function (orientation, attention, memory, language and visual-spatial skills) [doi: 10.1016/0022-3956(75)90026-6]. 
+More specific tasks/questions during the test: 
+1. What is the year? (wrong answer 0 points, right answer 1 point)
+2. What is the season? (wrong answer 0 points, right answer 1 point)
+3. What is the date? (wrong answer 0 points, right answer 1 point)
+4. What is the day of the week? (wrong answer 0 points, right answer 1 point)
+5. What is the month? (wrong answer 0 points, right answer 1 point)
+6. In what country we are now? (wrong answer 0 points, right answer 1 point)
+7. In what county we are now? (wrong answer 0 points, right answer 1 point)
+8. What is the name of this city? (wrong answer 0 points, right answer 1 point)
+9. What is this place where we are now? (wrong answer 0 points, right answer 1 point)
+10. In which floor we are now? (wrong answer 0 points, right answer 1 point)
+11. Soon I will say three words and you should memorize them and then repeat them after me. Words: shirt, brown and lively (or rose, ball and key) (max 3 points for right words in right order)
+12. I would like you to count backward from 100 by sevens (93, 86, 79, 72, 65) Stop after five answers. (93: 1 point, 86: 1 point, 79: 1 point, 72: 1 point, 65: 1 point, the examiner is allowed to repeat the question if the examinee does not understand it. If the examinee makes a mistake but continues with a right answer i.e. subtracts 7 from the wrong number, it equals to one wrong answer. No paper nor pencil is allowed)
+13. What were the words that I asked you to memorize and repeat? (max 3 points: right words &amp; order)
+14. What are the names of these two objects? (showing wrist watch and then pencil) (2 points for correct answers)
+15. Now I will read out loud one sentence, repeat after me: "No ifs, ands, or buts." (1 point for the perfect sentence)
+16. Now I will give you a paper and ask you to do following tasks: Take the paper in your left hand, fold it in half, and put it on your knees (max 3 points for performing all three tasks)
+17. Please read this text and do what it says (written text: close your eyes) (1 point if the examinee successfully reads the text and does what it says)
+18. Make up and write a sentence about anything. (1 point if the sentence is understandable and includes at least a subject and predicate, writing errors do not affect the score). 
+19. Please copy this picture (two pentagons). (1 point if all 10 angles are present and two must intersect resulting in a square in the middle of the pentagons)
+Maximal score: 30 points.</t>
+  </si>
+  <si>
+    <t>Maximal score 30 points.</t>
+  </si>
+  <si>
+    <t>psy_mci_moca_score</t>
+  </si>
+  <si>
+    <t>MoCa score</t>
+  </si>
+  <si>
+    <t>phy_walking</t>
+  </si>
+  <si>
+    <t>Walking for leisure</t>
+  </si>
+  <si>
+    <t>Frequency of walking for leisure per week</t>
+  </si>
+  <si>
+    <t>Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
+  </si>
+  <si>
+    <t>1 Less than once a week 
+2 1 to 5 times a week 
+3 6 times or more a week</t>
+  </si>
+  <si>
+    <t>The study collect frequency variables about "Walking or equivalent activity" and "Brisk walking or equivalent activity" that could include other type of low and moderate physical activity while the DataSchema variable is only about walking.</t>
+  </si>
+  <si>
+    <t>phy_occupational_pa</t>
+  </si>
+  <si>
+    <t>Occupational physical activity</t>
+  </si>
+  <si>
+    <t>Description of the typical physical activity required in the participant's occupation</t>
+  </si>
+  <si>
+    <t>1 Mostly sedentary-no physical demands
+2 Mostly standing or walking
+3 Standing and walking with lifting or carrying
+4 Strenuous physical work</t>
+  </si>
+  <si>
+    <t>phy_sport_participation</t>
+  </si>
+  <si>
+    <t>Sport participation</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant is participating in sport activity or not</t>
+  </si>
+  <si>
+    <t>When studies don't have a "other" category the "No" cannot be generated. In this situation only 1 and NA would be present. 
+Include any sport activity where the intensity was specified as being moderate or more.
+Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
+  </si>
+  <si>
+    <t>0 No 
+1 Yes</t>
+  </si>
+  <si>
+    <t>phy_active_commuting</t>
+  </si>
+  <si>
+    <t>Active commuting</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant is engaging in active commuting</t>
+  </si>
+  <si>
+    <t>Considered commuting when at least 15 minutes.</t>
+  </si>
+  <si>
+    <t>pacommuting1</t>
+  </si>
+  <si>
+    <t>Daily commuting to work</t>
+  </si>
+  <si>
+    <t>RPA_Transport</t>
+  </si>
+  <si>
+    <t>Daily commuting to work. Self-reported. Questionnaire item: How much time daily do you use commuting to work by walking, running or cycling? Response options: 1=No exercise while commuting, 2=1min-15min, 3=15min-less than half an hour, 4=half an hour-less than an hour, 5=hour or more, 6=I'm not working right now.</t>
+  </si>
+  <si>
+    <t>1=No exercise while commuting
+2=1min-15min
+3=15min-less than half an hour
+4=half an hour-less than an hour 
+5=hour or more
+6=I'm not working right now.</t>
+  </si>
+  <si>
+    <t>recode(1=0; 2=0; 3=1; 4=1; 5=1; 6=NA; ELSE=NA)</t>
+  </si>
+  <si>
+    <t>phy_leisure_time</t>
+  </si>
+  <si>
+    <t>Leisure-time physical activity, including sport</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant is engaging in physical activity during leisure-time (including sport)</t>
+  </si>
+  <si>
+    <t>Include any physical activity where the intensity was specified as being moderate (or equivalent) or more.
+Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
+  </si>
+  <si>
+    <t>pa_running1</t>
+  </si>
+  <si>
+    <t>weekly running or equivalent activity</t>
+  </si>
+  <si>
+    <t>RPA_Composite</t>
+  </si>
+  <si>
+    <t>Weekly running or equivalent activity. Self-reported. Questionnaire item: How much did you engage in following physical activities in a week during leisure time or commuting? 1. Running or equivalent activity. Response options for each of the physical activities: 1=Not at all, 2=Under ½ hour per week, 3=About an hour, 4=2-3 hours , 5=4 hours or more per week.</t>
+  </si>
+  <si>
+    <t>1 = Not at all 
+2 = Under ½ hour per week 
+3 = About an hour 
+4 = 2-3 hours 
+5 = 4 hours or more per week</t>
+  </si>
+  <si>
+    <t>The "No" responses was impossible to generate because the question was only about running or "equivalent activities".</t>
+  </si>
+  <si>
+    <t>recode(1=NA; 2=1; 3=1; 4=1; 5=1; ELSE=NA)</t>
+  </si>
+  <si>
+    <t>phy_mobility_limitation_SF36</t>
+  </si>
+  <si>
+    <t>Physical function SF36 subscale score</t>
+  </si>
+  <si>
+    <t>Total score of the physical function subscale of SF36</t>
+  </si>
+  <si>
+    <t>dis_vigorous1;
+dis_moderate1;
+dis_lift1;
+dis_climbseveral1;
+dis_climbone1;
+dis_bending1;
+dis_walk2km_1;
+dis_walk1km_1;
+dis_walk100m_1;
+dis_bath1</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>phy_SF36_nb_items</t>
+  </si>
+  <si>
+    <t>Number of non-missing items</t>
+  </si>
+  <si>
+    <t>Number of non-missing items in the SF36 physical function subscale</t>
+  </si>
+  <si>
+    <t>items</t>
+  </si>
+  <si>
+    <t>rowSums(mutate(.,
+temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
+temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
+temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
+temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
+temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
+temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
+temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
+temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
+temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
+temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
+select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
+temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
+na.rm = TRUE)) %&gt;%
+mutate(phy_SF36_nb_items = if_else(phy_SF36_nb_items == 0, NA, phy_SF36_nb_items)</t>
+  </si>
+  <si>
+    <t>Mlstr_harmo::comment</t>
+  </si>
+  <si>
+    <t>Mlstr_harmo::status</t>
+  </si>
+  <si>
+    <t>ifelse(rowSums(mutate(.,
+temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
+temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
+temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
+temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
+temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
+temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
+temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
+temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
+temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
+temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
+select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
+temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
+na.rm = TRUE) &lt; 5,NA,
+rowMeans(mutate(.,
+temp_dis_vigorous1 = 50 * dis_vigorous1 - 50, 
+temp_dis_moderate1 = 50 * dis_moderate1 - 50,
+temp_dis_lift1 = 50 * dis_lift1 - 50,
+temp_dis_climbseveral1 = 50 * dis_climbseveral1 - 50,
+temp_dis_climbone1 = 50 * dis_climbone1 - 50,
+temp_dis_bending1 = 50 * dis_bending1 - 50,
+temp_dis_walk2km_1 = 50 * dis_walk2km_1 - 50,
+temp_dis_walk1km_1 = 50 * dis_walk1km_1 - 50,
+temp_dis_walk100m_1 = 50 * dis_walk100m_1 - 50,
+temp_dis_bath1 = 50 * dis_bath1 - 50) %&gt;%
+select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
+temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
+na.rm = TRUE))</t>
+  </si>
+  <si>
+    <t>"FRA"</t>
   </si>
   <si>
     <t>case_when(
@@ -1761,14 +2536,14 @@
 !is.na(med8atc1) |
 !is.na(med9atc1)) &amp; 
 !grepl("^C02|^C03|^C07|^C08|^C09", med1atc1, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc2, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc3, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc4, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc5, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc6, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc7, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc8, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc9, ignore.case = TRUE) ~ 2L;
+!grepl("^C02|^C03|^C07|^C08|^C09", med2atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med3atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med4atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med5atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med6atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med7atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med8atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med9atc1, ignore.case = TRUE) ~ 2L;
 hypertension1 == 1 &amp;
 is.na(med1atc1) &amp;
 is.na(med2atc1) &amp;
@@ -1780,778 +2555,6 @@
 is.na(med8atc1) &amp;
 is.na(med9atc1) ~ 2L;
 ELSE ~ NA)</t>
-  </si>
-  <si>
-    <t>dis_msk_ever</t>
-  </si>
-  <si>
-    <t>Musculoskeletal diseases ever</t>
-  </si>
-  <si>
-    <t>Musculoskeletal diseases ever (osteoporosis, arthrosis, rheumatic disorder, osteoarthritis or rheumatism, rheumatoid arthritis, osteoarthritis, other arthritis, rheumatoid arthritis)</t>
-  </si>
-  <si>
-    <t>A "No" response can be assigned if the input variables were collected in Yes/No format. 
-If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
-  </si>
-  <si>
-    <t>osteoarthrosis1;
-osteoporosis1;
-sciatica1;
-rheumatoidarthritis1</t>
-  </si>
-  <si>
-    <t>Osteoarthrosis;
-Osteoporosis;
-Sciatica (lumbar disc herniation);
-Rheumatoid arthritis</t>
-  </si>
-  <si>
-    <t>HAM_LSI;HAM_LSI;HAM_LSI;HAM_LSI;HAM_LSI</t>
-  </si>
-  <si>
-    <t>Osteoarthrosis. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of osteoarthrosis? Response options: no, yes: previously, yes: currently;
-Osteoporosiss. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of osteoporosis? Response options: no, yes: previously, yes: currently;
-Sciatica (lumbar disc herniation). Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of sciatica (lumbar disc herniation)? Response options: no, yes: previously, yes: currently ;
-Fibromyalgia. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of fibromyalgia? Response options: no, yes: previously, yes: currently ;
-Rheumatoid arthritis. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of rheumatoid arthritis? Response options: no, yes: previously, yes: currently</t>
-  </si>
-  <si>
-    <t>Cohort profile: DOI: 10.1093/gerona/glaa193
-;Cohort profile: DOI: 10.1093/gerona/glaa193
-;Cohort profile: DOI: 10.1093/gerona/glaa193
-;Cohort profile: DOI: 10.1093/gerona/glaa193
-;Cohort profile: DOI: 10.1093/gerona/glaa193</t>
-  </si>
-  <si>
-    <t>case_when(
-osteoarthrosis1 %in% c(2, 3) | osteoporosis1 %in% c(2, 3) | sciatica1 %in% c(2, 3) | rheumatoidarthritis1 %in% c(2, 3) ~ 1L;
-osteoarthrosis1 == 1 &amp; osteoporosis1 == 1 &amp; sciatica1 == 1 &amp; rheumatoidarthritis1 == 1 ~ 0L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>dis_diabetes</t>
-  </si>
-  <si>
-    <t>Diabetes</t>
-  </si>
-  <si>
-    <t>Diabetes (including gestational diabetes and other types of diabetes but excluding impaired fasting glucose and impaired glucose tolerance)</t>
-  </si>
-  <si>
-    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
-If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned. 
-Add a harmonization comment about any study-specific wording for collecting information about diabetes (e.g., only Type 2 diabetes, excluding gestational diabetes).</t>
-  </si>
-  <si>
-    <t>diabetes1</t>
-  </si>
-  <si>
-    <t>Type 2 diabetes</t>
-  </si>
-  <si>
-    <t>Type 2 diabetes. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of type 2 diabetes? Response options: no, yes: previously, yes: currently.</t>
-  </si>
-  <si>
-    <t>1 = no 
-2 = yes, previously 
-3 = yes, currently</t>
-  </si>
-  <si>
-    <t>The study only ask about type 2 diabetes.</t>
-  </si>
-  <si>
-    <t>dis_diabetes_type</t>
-  </si>
-  <si>
-    <t>Diabetes type</t>
-  </si>
-  <si>
-    <t>Add a harmonization comment about any study-specific wording for collecting information about diabetes (e.g., only Type 2 diabetes collected).</t>
-  </si>
-  <si>
-    <t>1 Type 1 
-2 Type 2 
-3 Other</t>
-  </si>
-  <si>
-    <t>dis_cancer_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever</t>
-  </si>
-  <si>
-    <t>When studies do not have an "other cancer" category, a "No" cannot be generated. In this situation only 1 and NA would be present.
-Add a harmonization comment about any decisions made for harmonization.
-"Presumed no" can be specified only if a general cancer disease option is present in a select all that apply question where at least another option is selected but not this one.</t>
-  </si>
-  <si>
-    <t>malignanttumor1</t>
-  </si>
-  <si>
-    <t>Malignant tumor (cancer)</t>
-  </si>
-  <si>
-    <t>Malignant tumor (cancer). Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of malignant tumor? Response options: no, yes: previously, yes: currently</t>
-  </si>
-  <si>
-    <t>dis_cancer_bladder_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Bladder</t>
-  </si>
-  <si>
-    <t>The "No" response can be attributed only in 2 situations:
-- There is a parent variable about having any cancer, collected in Yes/No format.
-- The input variables were collected in Yes/No format for this specific cancer type
-If the input variables do not have a "No" response but are part of select all that apply section where at least another cancer type is selected, then a "Presumed no" can be assigned.</t>
-  </si>
-  <si>
-    <t>case_when(
-malignanttumor1 == 1 ~ 0L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>dis_cancer_breast_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Breast</t>
-  </si>
-  <si>
-    <t>dis_cancer_cervix_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Cervix</t>
-  </si>
-  <si>
-    <t>dis_cancer_colorectal_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Colon-Rectum</t>
-  </si>
-  <si>
-    <t>dis_cancer_kidney_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Kidney</t>
-  </si>
-  <si>
-    <t>dis_cancer_throat_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Throat/Larynx-Pharynx</t>
-  </si>
-  <si>
-    <t>dis_cancer_leukaemia_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Leukaemia</t>
-  </si>
-  <si>
-    <t>dis_cancer_lung_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Lung</t>
-  </si>
-  <si>
-    <t>dis_cancer_lymphoma_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Lymphoma</t>
-  </si>
-  <si>
-    <t>dis_cancer_prostate_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Prostate</t>
-  </si>
-  <si>
-    <t>dis_cancer_skin_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Skin</t>
-  </si>
-  <si>
-    <t>dis_cancer_stomach_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Stomach</t>
-  </si>
-  <si>
-    <t>dis_cancer_testicle_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Testicle</t>
-  </si>
-  <si>
-    <t>dis_cancer_uterus_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Uterus</t>
-  </si>
-  <si>
-    <t>dis_cancer_brain_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Brain</t>
-  </si>
-  <si>
-    <t>dis_cancer_liver_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Liver</t>
-  </si>
-  <si>
-    <t>dis_cancer_ovary_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Ovary</t>
-  </si>
-  <si>
-    <t>dis_cancer_pancreas_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Pancreas</t>
-  </si>
-  <si>
-    <t>dis_cancer_thyroid_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Thyroid</t>
-  </si>
-  <si>
-    <t>dis_hypercholesteromia_ever</t>
-  </si>
-  <si>
-    <t>Diagnosed hypercholesteromia</t>
-  </si>
-  <si>
-    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
-If the input variables do not have a "No" response but are part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
-  </si>
-  <si>
-    <t>highcholesterol1</t>
-  </si>
-  <si>
-    <t>High cholesterol</t>
-  </si>
-  <si>
-    <t>High cholesterol. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of high cholesterol? Response options: no, yes: previously, yes: currently.</t>
-  </si>
-  <si>
-    <t>dis_depression</t>
-  </si>
-  <si>
-    <t>Depression</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant has depression or not</t>
-  </si>
-  <si>
-    <t>Accept self-reported condition but with a note. 
-A "No" response can be assigned if the input variables were collected in Yes/No format.
-If the input variable do not have a "No" response but is part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
-  </si>
-  <si>
-    <t>depression1</t>
-  </si>
-  <si>
-    <t>depression</t>
-  </si>
-  <si>
-    <t>HAM_Depression</t>
-  </si>
-  <si>
-    <t>Depression. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of depression? Response options: no, yes: previously, yes: currently.</t>
-  </si>
-  <si>
-    <t>dis_alzheimers_dementia</t>
-  </si>
-  <si>
-    <t>Alzheimers/Dementia</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant has Alzheimers/Dementia</t>
-  </si>
-  <si>
-    <t>A "No" response can be assigned if the input variables were collected in Yes/No format.
-If the input variable do not have a "No" response but is part of select all that apply section where at least another condition is selected, then a "Presumed no" can be assigned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 Has not been diagnosed with Alzheimers or other dementia 
-1 Has been diagnosed with Alzheimers or other dementia 
-2 Has presumably not been diagnosed with Alzheimers or other dementia 
-</t>
-  </si>
-  <si>
-    <t>alzheimer1</t>
-  </si>
-  <si>
-    <t>Alzheimer or other dementia</t>
-  </si>
-  <si>
-    <t>HAM_Alzheimers</t>
-  </si>
-  <si>
-    <t>Alzheimer or other dementia. Self-reported. Questionnaire item: Has a doctor/physician given you a diagnosis of Alzheimer or other dementia? Response options: no, yes: previously, yes: currently.</t>
-  </si>
-  <si>
-    <t>med_lipid_lowering_cur</t>
-  </si>
-  <si>
-    <t>Current use of lipid lowering medication</t>
-  </si>
-  <si>
-    <t>Only include if lipid lowering medication is currently being taken. A "No" response is possible only if a Yes/No question is collected.
-If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
-  </si>
-  <si>
-    <t>med1atc1;
-med2atc1;
-med3atc1;
-med4atc1;
-med5atc1;
-med6atc1;
-med7atc1;
-med8atc1;
-med9atc1</t>
-  </si>
-  <si>
-    <t>Medication 1 to 5 atc code</t>
-  </si>
-  <si>
-    <t>HAM_MedUse</t>
-  </si>
-  <si>
-    <t>ATC code (Anatomical Therapeutic Chemical classification) of the medication used. Self-reported. Participants were asked to fill in a form names of medicines that they used. The full ATC code (A10BH01 etc). If the ATC code was not found, medicine was coded as follows: 
-X01= anti-hypertensive drug
-X02= diabetes drug
-X03= analgesic (painkiller)
-X04= cholesterol medicine
-X05= hormone replacement therapy
-X06= cortisone
-X07= vitamin 
-X08= nature cure/alternative remedy
-X10= something else/unspecified
-X11= antidepressant
-X12= allergy medicine
-X13= cortisone salve</t>
-  </si>
-  <si>
-    <t>ATC code (Anatomical Therapeutic Chemical classification)
-or if ATC code missing: 
-X01= anti-hypertensive drug
-X02= diabetes drug
-X03= analgesic (painkiller)
-X04= cholesterol medicine
-X05= hormone replacement therapy
-X06= cortisone
-X07= vitamin 
-X08= nature cure/alternative remedy
-X10= something else/unspecified
-X11= antidepressant
-X12= allergy medicine
-X13= cortisone salve</t>
-  </si>
-  <si>
-    <t>Derived from list of medication taken by the participant.</t>
-  </si>
-  <si>
-    <t>case_when(
-med1atc1 == "X04" ~ 1L;
-med2atc1 == "X04" ~ 1L;
-med3atc1 == "X04" ~ 1L;
-med4atc1 == "X04" ~ 1L;
-med5atc1 == "X04" ~ 1L;
-med6atc1 == "X04" ~ 1L;
-med7atc1 == "X04" ~ 1L;
-med8atc1 == "X04" ~ 1L;
-med9atc1 == "X04" ~ 1L;
-grepl("^C10", med1atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med2atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med3atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med4atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med5atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med6atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med7atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med8atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C10", med9atc1, ignore.case = TRUE) ~ 1L;
-!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>med_blood_pressure_cur</t>
-  </si>
-  <si>
-    <t>Current use of medication to manage blood pressure</t>
-  </si>
-  <si>
-    <t>Only include if medication for hypertension or high blood pressure is currently being taken. A "No" response is possible only if a Yes/No question is collected.
-The question must be separated from a hypertension or hbp diagnosis question.
-If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
-  </si>
-  <si>
-    <t>case_when(
-med1atc1 == "X01" ~ 1L;
-med2atc1 == "X01" ~ 1L;
-med3atc1 == "X01" ~ 1L;
-med4atc1 == "X01" ~ 1L;
-med5atc1 == "X01" ~ 1L;
-med6atc1 == "X01" ~ 1L;
-med7atc1 == "X01" ~ 1L;
-med8atc1 == "X01" ~ 1L;
-med9atc1 == "X01" ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med1atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med2atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med3atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med4atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med5atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med6atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med7atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med8atc1, ignore.case = TRUE) ~ 1L;
-grepl("^C02|^C03|^C07|^C08|^C09", med9atc1, ignore.case = TRUE) ~ 1L;
-!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>med_diabetes_cur</t>
-  </si>
-  <si>
-    <t>Current use of medication for diabetes</t>
-  </si>
-  <si>
-    <t>If the item is in a select all that apply where at least another item is selected then it is a "Presumed no".</t>
-  </si>
-  <si>
-    <t>case_when(
-med1atc1 == "X02" ~ 1L;
-med2atc1 == "X02" ~ 1L;
-med3atc1 == "X02" ~ 1L;
-med4atc1 == "X02" ~ 1L;
-med5atc1 == "X02" ~ 1L;
-med6atc1 == "X02" ~ 1L;
-med7atc1 == "X02" ~ 1L;
-med8atc1 == "X02" ~ 1L;
-med9atc1 == "X02" ~ 1L;
-grepl("^A10", med1atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med2atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med3atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med4atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med5atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med6atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med7atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med8atc1, ignore.case = TRUE) ~ 1L;
-grepl("^A10", med9atc1, ignore.case = TRUE) ~ 1L;
-!is.na(med1atc1) | !is.na(med2atc1) | !is.na(med3atc1) | !is.na(med4atc1) | !is.na(med5atc1) | !is.na(med6atc1) | !is.na(med7atc1) | !is.na(med8atc1) | !is.na(med9atc1) ~ 2L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>psy_dep_cesd20</t>
-  </si>
-  <si>
-    <t>CES-D (20 items) score</t>
-  </si>
-  <si>
-    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-60</t>
-  </si>
-  <si>
-    <t>psy_dep_cesd10</t>
-  </si>
-  <si>
-    <t>CES-D (10 items) score</t>
-  </si>
-  <si>
-    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-30</t>
-  </si>
-  <si>
-    <t>psy_dep_malaise</t>
-  </si>
-  <si>
-    <t>Malaise inventory (9 items) score</t>
-  </si>
-  <si>
-    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-24</t>
-  </si>
-  <si>
-    <t>psy_dep_kessler</t>
-  </si>
-  <si>
-    <t>Kessler psychological distress score</t>
-  </si>
-  <si>
-    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 10-50</t>
-  </si>
-  <si>
-    <t>psy_dep_phq9</t>
-  </si>
-  <si>
-    <t>PHQ-9 score</t>
-  </si>
-  <si>
-    <t>If the study has the total score variable, make sure the calculation is correct. Accepted score range is 0-27</t>
-  </si>
-  <si>
-    <t>psy_mci_mmse_score</t>
-  </si>
-  <si>
-    <t>MMSE score</t>
-  </si>
-  <si>
-    <t>mci1</t>
-  </si>
-  <si>
-    <t>Mild cognitive impairment</t>
-  </si>
-  <si>
-    <t>HAM_MildCI</t>
-  </si>
-  <si>
-    <t>Mild cognitive impairment was assessed during a clinical study visit with the Mini-Mental State Examination (MMSE) including items to assess cognitive function (orientation, attention, memory, language and visual-spatial skills) [doi: 10.1016/0022-3956(75)90026-6]. 
-More specific tasks/questions during the test: 
-1. What is the year? (wrong answer 0 points, right answer 1 point)
-2. What is the season? (wrong answer 0 points, right answer 1 point)
-3. What is the date? (wrong answer 0 points, right answer 1 point)
-4. What is the day of the week? (wrong answer 0 points, right answer 1 point)
-5. What is the month? (wrong answer 0 points, right answer 1 point)
-6. In what country we are now? (wrong answer 0 points, right answer 1 point)
-7. In what county we are now? (wrong answer 0 points, right answer 1 point)
-8. What is the name of this city? (wrong answer 0 points, right answer 1 point)
-9. What is this place where we are now? (wrong answer 0 points, right answer 1 point)
-10. In which floor we are now? (wrong answer 0 points, right answer 1 point)
-11. Soon I will say three words and you should memorize them and then repeat them after me. Words: shirt, brown and lively (or rose, ball and key) (max 3 points for right words in right order)
-12. I would like you to count backward from 100 by sevens (93, 86, 79, 72, 65) Stop after five answers. (93: 1 point, 86: 1 point, 79: 1 point, 72: 1 point, 65: 1 point, the examiner is allowed to repeat the question if the examinee does not understand it. If the examinee makes a mistake but continues with a right answer i.e. subtracts 7 from the wrong number, it equals to one wrong answer. No paper nor pencil is allowed)
-13. What were the words that I asked you to memorize and repeat? (max 3 points: right words &amp; order)
-14. What are the names of these two objects? (showing wrist watch and then pencil) (2 points for correct answers)
-15. Now I will read out loud one sentence, repeat after me: "No ifs, ands, or buts." (1 point for the perfect sentence)
-16. Now I will give you a paper and ask you to do following tasks: Take the paper in your left hand, fold it in half, and put it on your knees (max 3 points for performing all three tasks)
-17. Please read this text and do what it says (written text: close your eyes) (1 point if the examinee successfully reads the text and does what it says)
-18. Make up and write a sentence about anything. (1 point if the sentence is understandable and includes at least a subject and predicate, writing errors do not affect the score). 
-19. Please copy this picture (two pentagons). (1 point if all 10 angles are present and two must intersect resulting in a square in the middle of the pentagons)
-Maximal score: 30 points.</t>
-  </si>
-  <si>
-    <t>Maximal score 30 points.</t>
-  </si>
-  <si>
-    <t>psy_mci_moca_score</t>
-  </si>
-  <si>
-    <t>MoCa score</t>
-  </si>
-  <si>
-    <t>phy_walking</t>
-  </si>
-  <si>
-    <t>Walking for leisure</t>
-  </si>
-  <si>
-    <t>Frequency of walking for leisure per week</t>
-  </si>
-  <si>
-    <t>Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
-  </si>
-  <si>
-    <t>1 Less than once a week 
-2 1 to 5 times a week 
-3 6 times or more a week</t>
-  </si>
-  <si>
-    <t>The study collect frequency variables about "Walking or equivalent activity" and "Brisk walking or equivalent activity" that could include other type of low and moderate physical activity while the DataSchema variable is only about walking.</t>
-  </si>
-  <si>
-    <t>phy_occupational_pa</t>
-  </si>
-  <si>
-    <t>Occupational physical activity</t>
-  </si>
-  <si>
-    <t>Description of the typical physical activity required in the participant's occupation</t>
-  </si>
-  <si>
-    <t>1 Mostly sedentary-no physical demands
-2 Mostly standing or walking
-3 Standing and walking with lifting or carrying
-4 Strenuous physical work</t>
-  </si>
-  <si>
-    <t>phy_sport_participation</t>
-  </si>
-  <si>
-    <t>Sport participation</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is participating in sport activity or not</t>
-  </si>
-  <si>
-    <t>When studies don't have a "other" category the "No" cannot be generated. In this situation only 1 and NA would be present. 
-Include any sport activity where the intensity was specified as being moderate or more.
-Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
-  </si>
-  <si>
-    <t>0 No 
-1 Yes</t>
-  </si>
-  <si>
-    <t>phy_active_commuting</t>
-  </si>
-  <si>
-    <t>Active commuting</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is engaging in active commuting</t>
-  </si>
-  <si>
-    <t>Considered commuting when at least 15 minutes.</t>
-  </si>
-  <si>
-    <t>pacommuting1</t>
-  </si>
-  <si>
-    <t>Daily commuting to work</t>
-  </si>
-  <si>
-    <t>RPA_Transport</t>
-  </si>
-  <si>
-    <t>Daily commuting to work. Self-reported. Questionnaire item: How much time daily do you use commuting to work by walking, running or cycling? Response options: 1=No exercise while commuting, 2=1min-15min, 3=15min-less than half an hour, 4=half an hour-less than an hour, 5=hour or more, 6=I'm not working right now.</t>
-  </si>
-  <si>
-    <t>1=No exercise while commuting
-2=1min-15min
-3=15min-less than half an hour
-4=half an hour-less than an hour 
-5=hour or more
-6=I'm not working right now.</t>
-  </si>
-  <si>
-    <t>recode(1=0; 2=0; 3=1; 4=1; 5=1; 6=NA; ELSE=NA)</t>
-  </si>
-  <si>
-    <t>phy_leisure_time</t>
-  </si>
-  <si>
-    <t>Leisure-time physical activity, including sport</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is engaging in physical activity during leisure-time (including sport)</t>
-  </si>
-  <si>
-    <t>Include any physical activity where the intensity was specified as being moderate (or equivalent) or more.
-Add a harmonization comment about differences between study-specific variable and DataSchema variable in source, wording, and/or collection format.</t>
-  </si>
-  <si>
-    <t>pa_running1</t>
-  </si>
-  <si>
-    <t>weekly running or equivalent activity</t>
-  </si>
-  <si>
-    <t>RPA_Composite</t>
-  </si>
-  <si>
-    <t>Weekly running or equivalent activity. Self-reported. Questionnaire item: How much did you engage in following physical activities in a week during leisure time or commuting? 1. Running or equivalent activity. Response options for each of the physical activities: 1=Not at all, 2=Under ½ hour per week, 3=About an hour, 4=2-3 hours , 5=4 hours or more per week.</t>
-  </si>
-  <si>
-    <t>1 = Not at all 
-2 = Under ½ hour per week 
-3 = About an hour 
-4 = 2-3 hours 
-5 = 4 hours or more per week</t>
-  </si>
-  <si>
-    <t>The "No" responses was impossible to generate because the question was only about running or "equivalent activities".</t>
-  </si>
-  <si>
-    <t>recode(1=NA; 2=1; 3=1; 4=1; 5=1; ELSE=NA)</t>
-  </si>
-  <si>
-    <t>phy_mobility_limitation_SF36</t>
-  </si>
-  <si>
-    <t>Physical function SF36 subscale score</t>
-  </si>
-  <si>
-    <t>Total score of the physical function subscale of SF36</t>
-  </si>
-  <si>
-    <t>dis_vigorous1;
-dis_moderate1;
-dis_lift1;
-dis_climbseveral1;
-dis_climbone1;
-dis_bending1;
-dis_walk2km_1;
-dis_walk1km_1;
-dis_walk100m_1;
-dis_bath1</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>ifelse(rowSums(mutate(.,
-temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
-temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
-temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
-temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
-temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
-temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
-temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
-temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
-temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
-temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
-select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
-temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE)) &lt; 5,NA,
-rowMeans(mutate(.,
-temp_dis_vigorous1 = 50 * dis_vigorous1 - 50, 
-temp_dis_moderate1 = 50 * dis_moderate1 - 50,
-temp_dis_lift1 = 50 * dis_lift1 - 50,
-temp_dis_climbseveral1 = 50 * dis_climbseveral1 - 50,
-temp_dis_climbone1 = 50 * dis_climbone1 - 50,
-temp_dis_bending1 = 50 * dis_bending1 - 50,
-temp_dis_walk2km_1 = 50 * dis_walk2km_1 - 50,
-temp_dis_walk1km_1 = 50 * dis_walk1km_1 - 50,
-temp_dis_walk100m_1 = 50 * dis_walk100m_1 - 50,
-temp_dis_bath1 = 50 * dis_bath1 - 50) %&gt;%
-select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
-temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE))</t>
-  </si>
-  <si>
-    <t>phy_SF36_nb_items</t>
-  </si>
-  <si>
-    <t>Number of non-missing items</t>
-  </si>
-  <si>
-    <t>Number of non-missing items in the SF36 physical function subscale</t>
-  </si>
-  <si>
-    <t>items</t>
-  </si>
-  <si>
-    <t>rowSums(mutate(.,
-temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
-temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
-temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
-temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
-temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
-temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
-temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
-temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
-temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
-temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
-select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
-temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE)) %&gt;%
-mutate(phy_SF36_nb_items = if_else(phy_SF36_nb_items == 0, NA, phy_SF36_nb_items)</t>
-  </si>
-  <si>
-    <t>Mlstr_harmo::comment</t>
-  </si>
-  <si>
-    <t>Mlstr_harmo::status</t>
   </si>
 </sst>
 </file>
@@ -2928,6 +2931,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DD590CF-60F3-474A-8CF6-CAFB2AFA3E98}">
   <dimension ref="A1:X122"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="24" max="24" width="89.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -2988,10 +2994,10 @@
         <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="U1" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="V1" t="s">
         <v>19</v>
@@ -3088,13 +3094,13 @@
         <v>34</v>
       </c>
       <c r="V3" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="W3" t="s">
         <v>43</v>
       </c>
       <c r="X3" t="s">
-        <v>22</v>
+        <v>669</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -3126,13 +3132,13 @@
         <v>34</v>
       </c>
       <c r="V4" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="W4" t="s">
         <v>43</v>
       </c>
       <c r="X4" t="s">
-        <v>22</v>
+        <v>669</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -3164,7 +3170,7 @@
         <v>34</v>
       </c>
       <c r="V5" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="W5" t="s">
         <v>43</v>
@@ -3282,7 +3288,7 @@
         <v>42</v>
       </c>
       <c r="W7" t="s">
-        <v>61</v>
+        <v>127</v>
       </c>
       <c r="X7" t="s">
         <v>72</v>
@@ -6900,7 +6906,7 @@
         <v>420</v>
       </c>
       <c r="X79" s="1" t="s">
-        <v>486</v>
+        <v>670</v>
       </c>
     </row>
     <row r="80" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -6911,37 +6917,37 @@
         <v>22</v>
       </c>
       <c r="C80" t="s">
+        <v>486</v>
+      </c>
+      <c r="D80" t="s">
         <v>487</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>488</v>
-      </c>
-      <c r="E80" t="s">
-        <v>489</v>
       </c>
       <c r="F80" t="s">
         <v>49</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="J80" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K80" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="L80" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="L80" s="1" t="s">
+      <c r="M80" t="s">
         <v>492</v>
       </c>
-      <c r="M80" t="s">
+      <c r="N80" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="N80" s="1" t="s">
+      <c r="P80" s="1" t="s">
         <v>494</v>
-      </c>
-      <c r="P80" s="1" t="s">
-        <v>495</v>
       </c>
       <c r="Q80" t="s">
         <v>32</v>
@@ -6959,7 +6965,7 @@
         <v>420</v>
       </c>
       <c r="X80" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="81" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -6970,34 +6976,34 @@
         <v>22</v>
       </c>
       <c r="C81" t="s">
+        <v>496</v>
+      </c>
+      <c r="D81" t="s">
         <v>497</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>498</v>
-      </c>
-      <c r="E81" t="s">
-        <v>499</v>
       </c>
       <c r="F81" t="s">
         <v>49</v>
       </c>
       <c r="I81" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="J81" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K81" t="s">
+        <v>500</v>
+      </c>
+      <c r="L81" t="s">
         <v>501</v>
-      </c>
-      <c r="L81" t="s">
-        <v>502</v>
       </c>
       <c r="M81" t="s">
         <v>456</v>
       </c>
       <c r="N81" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="P81" t="s">
         <v>31</v>
@@ -7006,10 +7012,10 @@
         <v>32</v>
       </c>
       <c r="R81" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="T81" t="s">
         <v>504</v>
-      </c>
-      <c r="T81" t="s">
-        <v>505</v>
       </c>
       <c r="U81" t="s">
         <v>89</v>
@@ -7032,34 +7038,34 @@
         <v>22</v>
       </c>
       <c r="C82" t="s">
+        <v>505</v>
+      </c>
+      <c r="D82" t="s">
         <v>506</v>
       </c>
-      <c r="D82" t="s">
-        <v>507</v>
-      </c>
       <c r="E82" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F82" t="s">
         <v>49</v>
       </c>
       <c r="I82" t="s">
+        <v>507</v>
+      </c>
+      <c r="J82" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="J82" s="1" t="s">
-        <v>509</v>
-      </c>
       <c r="K82" t="s">
+        <v>500</v>
+      </c>
+      <c r="L82" t="s">
         <v>501</v>
-      </c>
-      <c r="L82" t="s">
-        <v>502</v>
       </c>
       <c r="M82" t="s">
         <v>456</v>
       </c>
       <c r="N82" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="P82" t="s">
         <v>31</v>
@@ -7068,10 +7074,10 @@
         <v>32</v>
       </c>
       <c r="R82" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="T82" t="s">
         <v>504</v>
-      </c>
-      <c r="T82" t="s">
-        <v>505</v>
       </c>
       <c r="U82" t="s">
         <v>89</v>
@@ -7094,34 +7100,34 @@
         <v>22</v>
       </c>
       <c r="C83" t="s">
+        <v>509</v>
+      </c>
+      <c r="D83" t="s">
         <v>510</v>
       </c>
-      <c r="D83" t="s">
-        <v>511</v>
-      </c>
       <c r="E83" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F83" t="s">
         <v>49</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J83" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K83" t="s">
+        <v>512</v>
+      </c>
+      <c r="L83" t="s">
         <v>513</v>
-      </c>
-      <c r="L83" t="s">
-        <v>514</v>
       </c>
       <c r="M83" t="s">
         <v>456</v>
       </c>
       <c r="N83" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P83" t="s">
         <v>31</v>
@@ -7130,7 +7136,7 @@
         <v>32</v>
       </c>
       <c r="R83" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U83" t="s">
         <v>34</v>
@@ -7153,34 +7159,34 @@
         <v>22</v>
       </c>
       <c r="C84" t="s">
+        <v>515</v>
+      </c>
+      <c r="D84" t="s">
         <v>516</v>
       </c>
-      <c r="D84" t="s">
-        <v>517</v>
-      </c>
       <c r="E84" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F84" t="s">
         <v>49</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J84" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K84" t="s">
+        <v>512</v>
+      </c>
+      <c r="L84" t="s">
         <v>513</v>
-      </c>
-      <c r="L84" t="s">
-        <v>514</v>
       </c>
       <c r="M84" t="s">
         <v>456</v>
       </c>
       <c r="N84" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P84" t="s">
         <v>31</v>
@@ -7189,7 +7195,7 @@
         <v>32</v>
       </c>
       <c r="R84" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U84" t="s">
         <v>34</v>
@@ -7201,7 +7207,7 @@
         <v>420</v>
       </c>
       <c r="X84" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="85" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7212,34 +7218,34 @@
         <v>22</v>
       </c>
       <c r="C85" t="s">
+        <v>519</v>
+      </c>
+      <c r="D85" t="s">
         <v>520</v>
       </c>
-      <c r="D85" t="s">
-        <v>521</v>
-      </c>
       <c r="E85" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="F85" t="s">
         <v>49</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J85" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K85" t="s">
+        <v>512</v>
+      </c>
+      <c r="L85" t="s">
         <v>513</v>
-      </c>
-      <c r="L85" t="s">
-        <v>514</v>
       </c>
       <c r="M85" t="s">
         <v>456</v>
       </c>
       <c r="N85" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P85" t="s">
         <v>31</v>
@@ -7248,7 +7254,7 @@
         <v>32</v>
       </c>
       <c r="R85" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U85" t="s">
         <v>34</v>
@@ -7260,7 +7266,7 @@
         <v>420</v>
       </c>
       <c r="X85" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="86" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7271,34 +7277,34 @@
         <v>22</v>
       </c>
       <c r="C86" t="s">
+        <v>521</v>
+      </c>
+      <c r="D86" t="s">
         <v>522</v>
       </c>
-      <c r="D86" t="s">
-        <v>523</v>
-      </c>
       <c r="E86" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F86" t="s">
         <v>49</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J86" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K86" t="s">
+        <v>512</v>
+      </c>
+      <c r="L86" t="s">
         <v>513</v>
-      </c>
-      <c r="L86" t="s">
-        <v>514</v>
       </c>
       <c r="M86" t="s">
         <v>456</v>
       </c>
       <c r="N86" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P86" t="s">
         <v>31</v>
@@ -7307,7 +7313,7 @@
         <v>32</v>
       </c>
       <c r="R86" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U86" t="s">
         <v>34</v>
@@ -7319,7 +7325,7 @@
         <v>420</v>
       </c>
       <c r="X86" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="87" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7330,34 +7336,34 @@
         <v>22</v>
       </c>
       <c r="C87" t="s">
+        <v>523</v>
+      </c>
+      <c r="D87" t="s">
         <v>524</v>
       </c>
-      <c r="D87" t="s">
-        <v>525</v>
-      </c>
       <c r="E87" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F87" t="s">
         <v>49</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J87" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K87" t="s">
+        <v>512</v>
+      </c>
+      <c r="L87" t="s">
         <v>513</v>
-      </c>
-      <c r="L87" t="s">
-        <v>514</v>
       </c>
       <c r="M87" t="s">
         <v>456</v>
       </c>
       <c r="N87" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P87" t="s">
         <v>31</v>
@@ -7366,7 +7372,7 @@
         <v>32</v>
       </c>
       <c r="R87" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U87" t="s">
         <v>34</v>
@@ -7378,7 +7384,7 @@
         <v>420</v>
       </c>
       <c r="X87" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="88" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7389,34 +7395,34 @@
         <v>22</v>
       </c>
       <c r="C88" t="s">
+        <v>525</v>
+      </c>
+      <c r="D88" t="s">
         <v>526</v>
       </c>
-      <c r="D88" t="s">
-        <v>527</v>
-      </c>
       <c r="E88" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F88" t="s">
         <v>49</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J88" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K88" t="s">
+        <v>512</v>
+      </c>
+      <c r="L88" t="s">
         <v>513</v>
-      </c>
-      <c r="L88" t="s">
-        <v>514</v>
       </c>
       <c r="M88" t="s">
         <v>456</v>
       </c>
       <c r="N88" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P88" t="s">
         <v>31</v>
@@ -7425,7 +7431,7 @@
         <v>32</v>
       </c>
       <c r="R88" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U88" t="s">
         <v>34</v>
@@ -7437,7 +7443,7 @@
         <v>420</v>
       </c>
       <c r="X88" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="89" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7448,34 +7454,34 @@
         <v>22</v>
       </c>
       <c r="C89" t="s">
+        <v>527</v>
+      </c>
+      <c r="D89" t="s">
         <v>528</v>
       </c>
-      <c r="D89" t="s">
-        <v>529</v>
-      </c>
       <c r="E89" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F89" t="s">
         <v>49</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J89" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K89" t="s">
+        <v>512</v>
+      </c>
+      <c r="L89" t="s">
         <v>513</v>
-      </c>
-      <c r="L89" t="s">
-        <v>514</v>
       </c>
       <c r="M89" t="s">
         <v>456</v>
       </c>
       <c r="N89" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P89" t="s">
         <v>31</v>
@@ -7484,7 +7490,7 @@
         <v>32</v>
       </c>
       <c r="R89" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U89" t="s">
         <v>34</v>
@@ -7496,7 +7502,7 @@
         <v>420</v>
       </c>
       <c r="X89" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="90" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7507,34 +7513,34 @@
         <v>22</v>
       </c>
       <c r="C90" t="s">
+        <v>529</v>
+      </c>
+      <c r="D90" t="s">
         <v>530</v>
       </c>
-      <c r="D90" t="s">
-        <v>531</v>
-      </c>
       <c r="E90" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F90" t="s">
         <v>49</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J90" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K90" t="s">
+        <v>512</v>
+      </c>
+      <c r="L90" t="s">
         <v>513</v>
-      </c>
-      <c r="L90" t="s">
-        <v>514</v>
       </c>
       <c r="M90" t="s">
         <v>456</v>
       </c>
       <c r="N90" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P90" t="s">
         <v>31</v>
@@ -7543,7 +7549,7 @@
         <v>32</v>
       </c>
       <c r="R90" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U90" t="s">
         <v>34</v>
@@ -7555,7 +7561,7 @@
         <v>420</v>
       </c>
       <c r="X90" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="91" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7566,34 +7572,34 @@
         <v>22</v>
       </c>
       <c r="C91" t="s">
+        <v>531</v>
+      </c>
+      <c r="D91" t="s">
         <v>532</v>
       </c>
-      <c r="D91" t="s">
-        <v>533</v>
-      </c>
       <c r="E91" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F91" t="s">
         <v>49</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J91" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K91" t="s">
+        <v>512</v>
+      </c>
+      <c r="L91" t="s">
         <v>513</v>
-      </c>
-      <c r="L91" t="s">
-        <v>514</v>
       </c>
       <c r="M91" t="s">
         <v>456</v>
       </c>
       <c r="N91" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P91" t="s">
         <v>31</v>
@@ -7602,7 +7608,7 @@
         <v>32</v>
       </c>
       <c r="R91" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U91" t="s">
         <v>34</v>
@@ -7614,7 +7620,7 @@
         <v>420</v>
       </c>
       <c r="X91" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="92" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7625,34 +7631,34 @@
         <v>22</v>
       </c>
       <c r="C92" t="s">
+        <v>533</v>
+      </c>
+      <c r="D92" t="s">
         <v>534</v>
       </c>
-      <c r="D92" t="s">
-        <v>535</v>
-      </c>
       <c r="E92" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F92" t="s">
         <v>49</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J92" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K92" t="s">
+        <v>512</v>
+      </c>
+      <c r="L92" t="s">
         <v>513</v>
-      </c>
-      <c r="L92" t="s">
-        <v>514</v>
       </c>
       <c r="M92" t="s">
         <v>456</v>
       </c>
       <c r="N92" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P92" t="s">
         <v>31</v>
@@ -7661,7 +7667,7 @@
         <v>32</v>
       </c>
       <c r="R92" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U92" t="s">
         <v>34</v>
@@ -7673,7 +7679,7 @@
         <v>420</v>
       </c>
       <c r="X92" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="93" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7684,34 +7690,34 @@
         <v>22</v>
       </c>
       <c r="C93" t="s">
+        <v>535</v>
+      </c>
+      <c r="D93" t="s">
         <v>536</v>
       </c>
-      <c r="D93" t="s">
-        <v>537</v>
-      </c>
       <c r="E93" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F93" t="s">
         <v>49</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J93" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K93" t="s">
+        <v>512</v>
+      </c>
+      <c r="L93" t="s">
         <v>513</v>
-      </c>
-      <c r="L93" t="s">
-        <v>514</v>
       </c>
       <c r="M93" t="s">
         <v>456</v>
       </c>
       <c r="N93" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P93" t="s">
         <v>31</v>
@@ -7720,7 +7726,7 @@
         <v>32</v>
       </c>
       <c r="R93" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U93" t="s">
         <v>34</v>
@@ -7732,7 +7738,7 @@
         <v>420</v>
       </c>
       <c r="X93" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="94" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7743,34 +7749,34 @@
         <v>22</v>
       </c>
       <c r="C94" t="s">
+        <v>537</v>
+      </c>
+      <c r="D94" t="s">
         <v>538</v>
       </c>
-      <c r="D94" t="s">
-        <v>539</v>
-      </c>
       <c r="E94" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F94" t="s">
         <v>49</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J94" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K94" t="s">
+        <v>512</v>
+      </c>
+      <c r="L94" t="s">
         <v>513</v>
-      </c>
-      <c r="L94" t="s">
-        <v>514</v>
       </c>
       <c r="M94" t="s">
         <v>456</v>
       </c>
       <c r="N94" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P94" t="s">
         <v>31</v>
@@ -7779,7 +7785,7 @@
         <v>32</v>
       </c>
       <c r="R94" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U94" t="s">
         <v>34</v>
@@ -7791,7 +7797,7 @@
         <v>420</v>
       </c>
       <c r="X94" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="95" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7802,34 +7808,34 @@
         <v>22</v>
       </c>
       <c r="C95" t="s">
+        <v>539</v>
+      </c>
+      <c r="D95" t="s">
         <v>540</v>
       </c>
-      <c r="D95" t="s">
-        <v>541</v>
-      </c>
       <c r="E95" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F95" t="s">
         <v>49</v>
       </c>
       <c r="I95" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J95" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K95" t="s">
+        <v>512</v>
+      </c>
+      <c r="L95" t="s">
         <v>513</v>
-      </c>
-      <c r="L95" t="s">
-        <v>514</v>
       </c>
       <c r="M95" t="s">
         <v>456</v>
       </c>
       <c r="N95" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P95" t="s">
         <v>31</v>
@@ -7838,7 +7844,7 @@
         <v>32</v>
       </c>
       <c r="R95" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U95" t="s">
         <v>34</v>
@@ -7850,7 +7856,7 @@
         <v>420</v>
       </c>
       <c r="X95" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="96" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7861,34 +7867,34 @@
         <v>22</v>
       </c>
       <c r="C96" t="s">
+        <v>541</v>
+      </c>
+      <c r="D96" t="s">
         <v>542</v>
       </c>
-      <c r="D96" t="s">
-        <v>543</v>
-      </c>
       <c r="E96" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F96" t="s">
         <v>49</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J96" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K96" t="s">
+        <v>512</v>
+      </c>
+      <c r="L96" t="s">
         <v>513</v>
-      </c>
-      <c r="L96" t="s">
-        <v>514</v>
       </c>
       <c r="M96" t="s">
         <v>456</v>
       </c>
       <c r="N96" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P96" t="s">
         <v>31</v>
@@ -7897,7 +7903,7 @@
         <v>32</v>
       </c>
       <c r="R96" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U96" t="s">
         <v>34</v>
@@ -7909,7 +7915,7 @@
         <v>420</v>
       </c>
       <c r="X96" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="97" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7920,34 +7926,34 @@
         <v>22</v>
       </c>
       <c r="C97" t="s">
+        <v>543</v>
+      </c>
+      <c r="D97" t="s">
         <v>544</v>
       </c>
-      <c r="D97" t="s">
-        <v>545</v>
-      </c>
       <c r="E97" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F97" t="s">
         <v>49</v>
       </c>
       <c r="I97" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J97" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K97" t="s">
+        <v>512</v>
+      </c>
+      <c r="L97" t="s">
         <v>513</v>
-      </c>
-      <c r="L97" t="s">
-        <v>514</v>
       </c>
       <c r="M97" t="s">
         <v>456</v>
       </c>
       <c r="N97" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P97" t="s">
         <v>31</v>
@@ -7956,7 +7962,7 @@
         <v>32</v>
       </c>
       <c r="R97" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U97" t="s">
         <v>34</v>
@@ -7968,7 +7974,7 @@
         <v>420</v>
       </c>
       <c r="X97" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="98" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -7979,34 +7985,34 @@
         <v>22</v>
       </c>
       <c r="C98" t="s">
+        <v>545</v>
+      </c>
+      <c r="D98" t="s">
         <v>546</v>
       </c>
-      <c r="D98" t="s">
-        <v>547</v>
-      </c>
       <c r="E98" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F98" t="s">
         <v>49</v>
       </c>
       <c r="I98" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J98" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K98" t="s">
+        <v>512</v>
+      </c>
+      <c r="L98" t="s">
         <v>513</v>
-      </c>
-      <c r="L98" t="s">
-        <v>514</v>
       </c>
       <c r="M98" t="s">
         <v>456</v>
       </c>
       <c r="N98" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P98" t="s">
         <v>31</v>
@@ -8015,7 +8021,7 @@
         <v>32</v>
       </c>
       <c r="R98" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U98" t="s">
         <v>34</v>
@@ -8027,7 +8033,7 @@
         <v>420</v>
       </c>
       <c r="X98" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="99" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8038,34 +8044,34 @@
         <v>22</v>
       </c>
       <c r="C99" t="s">
+        <v>547</v>
+      </c>
+      <c r="D99" t="s">
         <v>548</v>
       </c>
-      <c r="D99" t="s">
-        <v>549</v>
-      </c>
       <c r="E99" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F99" t="s">
         <v>49</v>
       </c>
       <c r="I99" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J99" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K99" t="s">
+        <v>512</v>
+      </c>
+      <c r="L99" t="s">
         <v>513</v>
-      </c>
-      <c r="L99" t="s">
-        <v>514</v>
       </c>
       <c r="M99" t="s">
         <v>456</v>
       </c>
       <c r="N99" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P99" t="s">
         <v>31</v>
@@ -8074,7 +8080,7 @@
         <v>32</v>
       </c>
       <c r="R99" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U99" t="s">
         <v>34</v>
@@ -8086,7 +8092,7 @@
         <v>420</v>
       </c>
       <c r="X99" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="100" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8097,34 +8103,34 @@
         <v>22</v>
       </c>
       <c r="C100" t="s">
+        <v>549</v>
+      </c>
+      <c r="D100" t="s">
         <v>550</v>
       </c>
-      <c r="D100" t="s">
-        <v>551</v>
-      </c>
       <c r="E100" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F100" t="s">
         <v>49</v>
       </c>
       <c r="I100" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J100" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K100" t="s">
+        <v>512</v>
+      </c>
+      <c r="L100" t="s">
         <v>513</v>
-      </c>
-      <c r="L100" t="s">
-        <v>514</v>
       </c>
       <c r="M100" t="s">
         <v>456</v>
       </c>
       <c r="N100" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P100" t="s">
         <v>31</v>
@@ -8133,7 +8139,7 @@
         <v>32</v>
       </c>
       <c r="R100" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U100" t="s">
         <v>34</v>
@@ -8145,7 +8151,7 @@
         <v>420</v>
       </c>
       <c r="X100" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="101" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8156,34 +8162,34 @@
         <v>22</v>
       </c>
       <c r="C101" t="s">
+        <v>551</v>
+      </c>
+      <c r="D101" t="s">
         <v>552</v>
       </c>
-      <c r="D101" t="s">
-        <v>553</v>
-      </c>
       <c r="E101" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="F101" t="s">
         <v>49</v>
       </c>
       <c r="I101" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J101" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K101" t="s">
+        <v>512</v>
+      </c>
+      <c r="L101" t="s">
         <v>513</v>
-      </c>
-      <c r="L101" t="s">
-        <v>514</v>
       </c>
       <c r="M101" t="s">
         <v>456</v>
       </c>
       <c r="N101" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P101" t="s">
         <v>31</v>
@@ -8192,7 +8198,7 @@
         <v>32</v>
       </c>
       <c r="R101" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U101" t="s">
         <v>34</v>
@@ -8204,7 +8210,7 @@
         <v>420</v>
       </c>
       <c r="X101" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="102" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8215,34 +8221,34 @@
         <v>22</v>
       </c>
       <c r="C102" t="s">
+        <v>553</v>
+      </c>
+      <c r="D102" t="s">
         <v>554</v>
       </c>
-      <c r="D102" t="s">
-        <v>555</v>
-      </c>
       <c r="E102" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F102" t="s">
         <v>49</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J102" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K102" t="s">
+        <v>512</v>
+      </c>
+      <c r="L102" t="s">
         <v>513</v>
-      </c>
-      <c r="L102" t="s">
-        <v>514</v>
       </c>
       <c r="M102" t="s">
         <v>456</v>
       </c>
       <c r="N102" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="P102" t="s">
         <v>31</v>
@@ -8251,7 +8257,7 @@
         <v>32</v>
       </c>
       <c r="R102" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U102" t="s">
         <v>34</v>
@@ -8263,7 +8269,7 @@
         <v>420</v>
       </c>
       <c r="X102" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="103" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8274,34 +8280,34 @@
         <v>22</v>
       </c>
       <c r="C103" t="s">
+        <v>555</v>
+      </c>
+      <c r="D103" t="s">
         <v>556</v>
       </c>
-      <c r="D103" t="s">
-        <v>557</v>
-      </c>
       <c r="E103" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F103" t="s">
         <v>49</v>
       </c>
       <c r="I103" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J103" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K103" t="s">
+        <v>558</v>
+      </c>
+      <c r="L103" t="s">
         <v>559</v>
-      </c>
-      <c r="L103" t="s">
-        <v>560</v>
       </c>
       <c r="M103" t="s">
         <v>456</v>
       </c>
       <c r="N103" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="P103" t="s">
         <v>31</v>
@@ -8310,7 +8316,7 @@
         <v>32</v>
       </c>
       <c r="R103" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U103" t="s">
         <v>34</v>
@@ -8333,34 +8339,34 @@
         <v>22</v>
       </c>
       <c r="C104" t="s">
+        <v>561</v>
+      </c>
+      <c r="D104" t="s">
         <v>562</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>563</v>
-      </c>
-      <c r="E104" t="s">
-        <v>564</v>
       </c>
       <c r="F104" t="s">
         <v>49</v>
       </c>
       <c r="I104" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="J104" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K104" t="s">
+        <v>565</v>
+      </c>
+      <c r="L104" t="s">
         <v>566</v>
       </c>
-      <c r="L104" t="s">
+      <c r="M104" t="s">
         <v>567</v>
       </c>
-      <c r="M104" t="s">
+      <c r="N104" t="s">
         <v>568</v>
-      </c>
-      <c r="N104" t="s">
-        <v>569</v>
       </c>
       <c r="P104" t="s">
         <v>31</v>
@@ -8369,7 +8375,7 @@
         <v>32</v>
       </c>
       <c r="R104" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U104" t="s">
         <v>34</v>
@@ -8392,34 +8398,34 @@
         <v>22</v>
       </c>
       <c r="C105" t="s">
+        <v>569</v>
+      </c>
+      <c r="D105" t="s">
         <v>570</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>571</v>
-      </c>
-      <c r="E105" t="s">
-        <v>572</v>
       </c>
       <c r="F105" t="s">
         <v>49</v>
       </c>
       <c r="I105" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="J105" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="J105" s="1" t="s">
+      <c r="K105" t="s">
         <v>574</v>
       </c>
-      <c r="K105" t="s">
+      <c r="L105" t="s">
         <v>575</v>
       </c>
-      <c r="L105" t="s">
+      <c r="M105" t="s">
         <v>576</v>
       </c>
-      <c r="M105" t="s">
+      <c r="N105" t="s">
         <v>577</v>
-      </c>
-      <c r="N105" t="s">
-        <v>578</v>
       </c>
       <c r="P105" t="s">
         <v>31</v>
@@ -8428,7 +8434,7 @@
         <v>32</v>
       </c>
       <c r="R105" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="U105" t="s">
         <v>34</v>
@@ -8451,34 +8457,34 @@
         <v>22</v>
       </c>
       <c r="C106" t="s">
+        <v>578</v>
+      </c>
+      <c r="D106" t="s">
         <v>579</v>
       </c>
-      <c r="D106" t="s">
-        <v>580</v>
-      </c>
       <c r="E106" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F106" t="s">
         <v>49</v>
       </c>
       <c r="I106" s="1" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="J106" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K106" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="L106" t="s">
         <v>582</v>
       </c>
-      <c r="L106" t="s">
+      <c r="M106" t="s">
         <v>583</v>
       </c>
-      <c r="M106" t="s">
+      <c r="N106" s="1" t="s">
         <v>584</v>
-      </c>
-      <c r="N106" s="1" t="s">
-        <v>585</v>
       </c>
       <c r="P106" t="s">
         <v>31</v>
@@ -8487,10 +8493,10 @@
         <v>32</v>
       </c>
       <c r="R106" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="T106" t="s">
         <v>586</v>
-      </c>
-      <c r="T106" t="s">
-        <v>587</v>
       </c>
       <c r="U106" t="s">
         <v>34</v>
@@ -8502,7 +8508,7 @@
         <v>420</v>
       </c>
       <c r="X106" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="107" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8513,34 +8519,34 @@
         <v>22</v>
       </c>
       <c r="C107" t="s">
+        <v>588</v>
+      </c>
+      <c r="D107" t="s">
         <v>589</v>
       </c>
-      <c r="D107" t="s">
-        <v>590</v>
-      </c>
       <c r="E107" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F107" t="s">
         <v>49</v>
       </c>
       <c r="I107" s="1" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="J107" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K107" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="L107" t="s">
         <v>582</v>
       </c>
-      <c r="L107" t="s">
+      <c r="M107" t="s">
         <v>583</v>
       </c>
-      <c r="M107" t="s">
+      <c r="N107" s="1" t="s">
         <v>584</v>
-      </c>
-      <c r="N107" s="1" t="s">
-        <v>585</v>
       </c>
       <c r="P107" t="s">
         <v>31</v>
@@ -8549,10 +8555,10 @@
         <v>32</v>
       </c>
       <c r="R107" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="T107" t="s">
         <v>586</v>
-      </c>
-      <c r="T107" t="s">
-        <v>587</v>
       </c>
       <c r="U107" t="s">
         <v>34</v>
@@ -8564,7 +8570,7 @@
         <v>420</v>
       </c>
       <c r="X107" s="1" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="108" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -8575,34 +8581,34 @@
         <v>22</v>
       </c>
       <c r="C108" t="s">
+        <v>592</v>
+      </c>
+      <c r="D108" t="s">
         <v>593</v>
       </c>
-      <c r="D108" t="s">
-        <v>594</v>
-      </c>
       <c r="E108" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F108" t="s">
         <v>49</v>
       </c>
       <c r="I108" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="J108" s="1" t="s">
         <v>436</v>
       </c>
       <c r="K108" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="L108" t="s">
         <v>582</v>
       </c>
-      <c r="L108" t="s">
+      <c r="M108" t="s">
         <v>583</v>
       </c>
-      <c r="M108" t="s">
+      <c r="N108" s="1" t="s">
         <v>584</v>
-      </c>
-      <c r="N108" s="1" t="s">
-        <v>585</v>
       </c>
       <c r="P108" t="s">
         <v>31</v>
@@ -8611,10 +8617,10 @@
         <v>32</v>
       </c>
       <c r="R108" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="T108" t="s">
         <v>586</v>
-      </c>
-      <c r="T108" t="s">
-        <v>587</v>
       </c>
       <c r="U108" t="s">
         <v>34</v>
@@ -8626,7 +8632,7 @@
         <v>420</v>
       </c>
       <c r="X108" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="109" spans="1:24" x14ac:dyDescent="0.25">
@@ -8637,19 +8643,19 @@
         <v>22</v>
       </c>
       <c r="C109" t="s">
+        <v>596</v>
+      </c>
+      <c r="D109" t="s">
         <v>597</v>
       </c>
-      <c r="D109" t="s">
-        <v>598</v>
-      </c>
       <c r="E109" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="F109" t="s">
         <v>49</v>
       </c>
       <c r="I109" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="K109" t="s">
         <v>41</v>
@@ -8675,19 +8681,19 @@
         <v>22</v>
       </c>
       <c r="C110" t="s">
+        <v>599</v>
+      </c>
+      <c r="D110" t="s">
         <v>600</v>
       </c>
-      <c r="D110" t="s">
-        <v>601</v>
-      </c>
       <c r="E110" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F110" t="s">
         <v>49</v>
       </c>
       <c r="I110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="K110" t="s">
         <v>41</v>
@@ -8713,19 +8719,19 @@
         <v>22</v>
       </c>
       <c r="C111" t="s">
+        <v>602</v>
+      </c>
+      <c r="D111" t="s">
         <v>603</v>
       </c>
-      <c r="D111" t="s">
-        <v>604</v>
-      </c>
       <c r="E111" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F111" t="s">
         <v>49</v>
       </c>
       <c r="I111" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="K111" t="s">
         <v>41</v>
@@ -8751,19 +8757,19 @@
         <v>22</v>
       </c>
       <c r="C112" t="s">
+        <v>605</v>
+      </c>
+      <c r="D112" t="s">
         <v>606</v>
       </c>
-      <c r="D112" t="s">
-        <v>607</v>
-      </c>
       <c r="E112" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F112" t="s">
         <v>49</v>
       </c>
       <c r="I112" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="K112" t="s">
         <v>41</v>
@@ -8789,19 +8795,19 @@
         <v>22</v>
       </c>
       <c r="C113" t="s">
+        <v>608</v>
+      </c>
+      <c r="D113" t="s">
         <v>609</v>
       </c>
-      <c r="D113" t="s">
-        <v>610</v>
-      </c>
       <c r="E113" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F113" t="s">
         <v>49</v>
       </c>
       <c r="I113" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="K113" t="s">
         <v>41</v>
@@ -8827,31 +8833,31 @@
         <v>22</v>
       </c>
       <c r="C114" t="s">
+        <v>611</v>
+      </c>
+      <c r="D114" t="s">
         <v>612</v>
       </c>
-      <c r="D114" t="s">
-        <v>613</v>
-      </c>
       <c r="E114" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F114" t="s">
         <v>49</v>
       </c>
       <c r="I114" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="K114" t="s">
+        <v>613</v>
+      </c>
+      <c r="L114" t="s">
         <v>614</v>
       </c>
-      <c r="L114" t="s">
+      <c r="M114" t="s">
         <v>615</v>
       </c>
-      <c r="M114" t="s">
+      <c r="N114" s="1" t="s">
         <v>616</v>
-      </c>
-      <c r="N114" s="1" t="s">
-        <v>617</v>
       </c>
       <c r="P114" t="s">
         <v>31</v>
@@ -8860,7 +8866,7 @@
         <v>82</v>
       </c>
       <c r="R114" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="U114" t="s">
         <v>34</v>
@@ -8883,19 +8889,19 @@
         <v>22</v>
       </c>
       <c r="C115" t="s">
+        <v>618</v>
+      </c>
+      <c r="D115" t="s">
         <v>619</v>
       </c>
-      <c r="D115" t="s">
-        <v>620</v>
-      </c>
       <c r="E115" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F115" t="s">
         <v>49</v>
       </c>
       <c r="I115" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="K115" t="s">
         <v>41</v>
@@ -8921,28 +8927,28 @@
         <v>22</v>
       </c>
       <c r="C116" t="s">
+        <v>620</v>
+      </c>
+      <c r="D116" t="s">
         <v>621</v>
       </c>
-      <c r="D116" t="s">
+      <c r="E116" t="s">
         <v>622</v>
-      </c>
-      <c r="E116" t="s">
-        <v>623</v>
       </c>
       <c r="F116" t="s">
         <v>49</v>
       </c>
       <c r="I116" t="s">
+        <v>623</v>
+      </c>
+      <c r="J116" s="1" t="s">
         <v>624</v>
-      </c>
-      <c r="J116" s="1" t="s">
-        <v>625</v>
       </c>
       <c r="K116" t="s">
         <v>41</v>
       </c>
       <c r="T116" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="U116" t="s">
         <v>89</v>
@@ -8965,22 +8971,22 @@
         <v>22</v>
       </c>
       <c r="C117" t="s">
+        <v>626</v>
+      </c>
+      <c r="D117" t="s">
         <v>627</v>
       </c>
-      <c r="D117" t="s">
+      <c r="E117" t="s">
         <v>628</v>
-      </c>
-      <c r="E117" t="s">
-        <v>629</v>
       </c>
       <c r="F117" t="s">
         <v>49</v>
       </c>
       <c r="I117" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J117" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="K117" t="s">
         <v>41</v>
@@ -9006,22 +9012,22 @@
         <v>22</v>
       </c>
       <c r="C118" t="s">
+        <v>630</v>
+      </c>
+      <c r="D118" t="s">
         <v>631</v>
       </c>
-      <c r="D118" t="s">
+      <c r="E118" t="s">
         <v>632</v>
-      </c>
-      <c r="E118" t="s">
-        <v>633</v>
       </c>
       <c r="F118" t="s">
         <v>49</v>
       </c>
       <c r="I118" s="1" t="s">
+        <v>633</v>
+      </c>
+      <c r="J118" s="1" t="s">
         <v>634</v>
-      </c>
-      <c r="J118" s="1" t="s">
-        <v>635</v>
       </c>
       <c r="K118" t="s">
         <v>41</v>
@@ -9047,34 +9053,34 @@
         <v>22</v>
       </c>
       <c r="C119" t="s">
+        <v>635</v>
+      </c>
+      <c r="D119" t="s">
         <v>636</v>
       </c>
-      <c r="D119" t="s">
+      <c r="E119" t="s">
         <v>637</v>
-      </c>
-      <c r="E119" t="s">
-        <v>638</v>
       </c>
       <c r="F119" t="s">
         <v>49</v>
       </c>
       <c r="I119" t="s">
+        <v>638</v>
+      </c>
+      <c r="J119" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="K119" t="s">
         <v>639</v>
       </c>
-      <c r="J119" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="K119" t="s">
+      <c r="L119" t="s">
         <v>640</v>
       </c>
-      <c r="L119" t="s">
+      <c r="M119" t="s">
         <v>641</v>
       </c>
-      <c r="M119" t="s">
+      <c r="N119" t="s">
         <v>642</v>
-      </c>
-      <c r="N119" t="s">
-        <v>643</v>
       </c>
       <c r="P119" t="s">
         <v>31</v>
@@ -9083,7 +9089,7 @@
         <v>32</v>
       </c>
       <c r="R119" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="U119" t="s">
         <v>34</v>
@@ -9095,7 +9101,7 @@
         <v>127</v>
       </c>
       <c r="X119" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="120" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -9106,34 +9112,34 @@
         <v>22</v>
       </c>
       <c r="C120" t="s">
+        <v>645</v>
+      </c>
+      <c r="D120" t="s">
         <v>646</v>
       </c>
-      <c r="D120" t="s">
+      <c r="E120" t="s">
         <v>647</v>
-      </c>
-      <c r="E120" t="s">
-        <v>648</v>
       </c>
       <c r="F120" t="s">
         <v>49</v>
       </c>
       <c r="I120" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="J120" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="K120" t="s">
         <v>649</v>
       </c>
-      <c r="J120" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="K120" t="s">
+      <c r="L120" t="s">
         <v>650</v>
       </c>
-      <c r="L120" t="s">
+      <c r="M120" t="s">
         <v>651</v>
       </c>
-      <c r="M120" t="s">
+      <c r="N120" t="s">
         <v>652</v>
-      </c>
-      <c r="N120" t="s">
-        <v>653</v>
       </c>
       <c r="P120" t="s">
         <v>31</v>
@@ -9142,10 +9148,10 @@
         <v>32</v>
       </c>
       <c r="R120" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="T120" t="s">
         <v>654</v>
-      </c>
-      <c r="T120" t="s">
-        <v>655</v>
       </c>
       <c r="U120" t="s">
         <v>34</v>
@@ -9157,7 +9163,7 @@
         <v>127</v>
       </c>
       <c r="X120" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="121" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
@@ -9168,19 +9174,19 @@
         <v>22</v>
       </c>
       <c r="C121" t="s">
+        <v>656</v>
+      </c>
+      <c r="D121" t="s">
         <v>657</v>
       </c>
-      <c r="D121" t="s">
+      <c r="E121" t="s">
         <v>658</v>
-      </c>
-      <c r="E121" t="s">
-        <v>659</v>
       </c>
       <c r="F121" t="s">
         <v>138</v>
       </c>
       <c r="K121" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="U121" t="s">
         <v>34</v>
@@ -9189,13 +9195,13 @@
         <v>42</v>
       </c>
       <c r="W121" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="X121" s="1" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="122" spans="1:24" ht="409.5" x14ac:dyDescent="0.25">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="122" spans="1:24" ht="270" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -9203,22 +9209,22 @@
         <v>22</v>
       </c>
       <c r="C122" t="s">
+        <v>661</v>
+      </c>
+      <c r="D122" t="s">
+        <v>662</v>
+      </c>
+      <c r="E122" t="s">
         <v>663</v>
-      </c>
-      <c r="D122" t="s">
-        <v>664</v>
-      </c>
-      <c r="E122" t="s">
-        <v>665</v>
       </c>
       <c r="F122" t="s">
         <v>49</v>
       </c>
       <c r="G122" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="K122" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="U122" t="s">
         <v>34</v>
@@ -9230,7 +9236,7 @@
         <v>61</v>
       </c>
       <c r="X122" s="1" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct dis hbp diag med harmo rule
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-FRA.xlsx
+++ b/baseline/data_processing_elements-FRA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\FRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E32CC9-4B21-4B0E-B4D4-12415C205242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F9DE9E-7778-42D0-A571-A191D0FC2144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CCDECE63-0FFC-4822-923F-34FACAF497E3}"/>
   </bookViews>
@@ -2508,14 +2508,14 @@
 med8atc1 != "X01"&amp;
 med9atc1 != "X01" &amp;
 !grepl("^C02|^C03|^C07|^C08|^C09", med1atc1, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc2, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc3, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc4, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc5, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc6, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc7, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc8, ignore.case = TRUE) &amp;
-!grepl("^C02|^C03|^C07|^C08|^C09", med1atc9, ignore.case = TRUE) ~ 0L;
+!grepl("^C02|^C03|^C07|^C08|^C09", med2atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med3atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med4atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med5atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med6atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med7atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med8atc1, ignore.case = TRUE) &amp;
+!grepl("^C02|^C03|^C07|^C08|^C09", med9atc1, ignore.case = TRUE) ~ 0L;
 is.na(hypertension1) &amp;
 med1atc1 != "X01" &amp;
 med2atc1 != "X01" &amp;

</xml_diff>

<commit_message>
correct SF36 n items variable algorithm
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-FRA.xlsx
+++ b/baseline/data_processing_elements-FRA.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF48816-2EFE-4463-8AC6-C514F138B51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CF1CCA-1863-4B33-A3BC-34CA21583BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CCDECE63-0FFC-4822-923F-34FACAF497E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$Z$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1647,23 +1650,6 @@
   </si>
   <si>
     <t>items</t>
-  </si>
-  <si>
-    <t>rowSums(mutate(.,
-temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
-temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
-temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
-temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
-temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
-temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
-temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
-temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
-temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
-temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
-select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
-temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE)) %&gt;%
-mutate(phy_SF36_nb_items = if_else(phy_SF36_nb_items == 0, NA, phy_SF36_nb_items)</t>
   </si>
   <si>
     <t>Mlstr_harmo::comment</t>
@@ -2770,6 +2756,36 @@
   </si>
   <si>
     <t>cog_mci_moca</t>
+  </si>
+  <si>
+    <t>ifelse( rowSums(mutate(.,
+temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
+temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
+temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
+temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
+temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
+temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
+temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
+temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
+temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
+temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
+select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
+temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
+na.rm = TRUE)) == 0,NA,
+rowSums(mutate(.,
+temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
+temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
+temp_dis_lift1 = as.numeric(!is.na(dis_lift1)),
+temp_dis_climbseveral1 = as.numeric(!is.na(dis_climbseveral1)),
+temp_dis_climbone1 = as.numeric(!is.na(dis_climbone1)),
+temp_dis_bending1 = as.numeric(!is.na(dis_bending1)),
+temp_dis_walk2km_1 = as.numeric(!is.na(dis_walk2km_1)),
+temp_dis_walk1km_1 = as.numeric(!is.na(dis_walk1km_1)),
+temp_dis_walk100m_1 = as.numeric(!is.na(dis_walk100m_1)),
+temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
+select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
+temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
+na.rm = TRUE)))</t>
   </si>
 </sst>
 </file>
@@ -3179,6 +3195,7 @@
     <col min="5" max="5" width="57.5703125" customWidth="1"/>
     <col min="10" max="10" width="48.7109375" customWidth="1"/>
     <col min="12" max="12" width="26.5703125" customWidth="1"/>
+    <col min="13" max="13" width="41.42578125" customWidth="1"/>
     <col min="26" max="26" width="89.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3241,10 +3258,10 @@
         <v>18</v>
       </c>
       <c r="V1" t="s">
+        <v>447</v>
+      </c>
+      <c r="W1" t="s">
         <v>448</v>
-      </c>
-      <c r="W1" t="s">
-        <v>449</v>
       </c>
       <c r="X1" t="s">
         <v>19</v>
@@ -3264,13 +3281,13 @@
         <v>22</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>23</v>
@@ -3279,7 +3296,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -3331,7 +3348,7 @@
         <v>35</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>23</v>
@@ -3340,7 +3357,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="3"/>
@@ -3357,7 +3374,7 @@
         <v>38</v>
       </c>
       <c r="Z3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="135" x14ac:dyDescent="0.25">
@@ -3374,7 +3391,7 @@
         <v>40</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>23</v>
@@ -3383,7 +3400,7 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="3"/>
@@ -3400,7 +3417,7 @@
         <v>38</v>
       </c>
       <c r="Z4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -3417,7 +3434,7 @@
         <v>42</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>43</v>
@@ -3426,7 +3443,7 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="3"/>
@@ -3457,7 +3474,7 @@
         <v>44</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>45</v>
@@ -3471,10 +3488,10 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>463</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>464</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" t="s">
@@ -3536,7 +3553,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="M7" t="s">
         <v>57</v>
@@ -3586,7 +3603,7 @@
         <v>64</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>43</v>
@@ -3597,10 +3614,10 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>467</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>468</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" t="s">
@@ -3645,13 +3662,13 @@
         <v>22</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>72</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>43</v>
@@ -3660,13 +3677,13 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>471</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>472</v>
       </c>
       <c r="M9" t="s">
         <v>36</v>
@@ -3692,7 +3709,7 @@
         <v>22</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>75</v>
@@ -3707,13 +3724,13 @@
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="K10" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>471</v>
-      </c>
       <c r="L10" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M10" t="s">
         <v>36</v>
@@ -3745,7 +3762,7 @@
         <v>78</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>43</v>
@@ -3753,16 +3770,16 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>477</v>
-      </c>
       <c r="L11" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M11" t="s">
         <v>36</v>
@@ -3791,10 +3808,10 @@
         <v>79</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>478</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>479</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>43</v>
@@ -3802,16 +3819,16 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>481</v>
-      </c>
       <c r="K12" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M12" t="s">
         <v>36</v>
@@ -3843,7 +3860,7 @@
         <v>81</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>43</v>
@@ -3851,16 +3868,16 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="J13" s="2" t="s">
-        <v>484</v>
-      </c>
       <c r="K13" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M13" t="s">
         <v>36</v>
@@ -3892,7 +3909,7 @@
         <v>83</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>43</v>
@@ -3900,16 +3917,16 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>487</v>
-      </c>
       <c r="K14" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M14" t="s">
         <v>36</v>
@@ -3941,7 +3958,7 @@
         <v>85</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>43</v>
@@ -3949,16 +3966,16 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="J15" s="2" t="s">
-        <v>490</v>
-      </c>
       <c r="K15" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M15" t="s">
         <v>36</v>
@@ -3990,7 +4007,7 @@
         <v>87</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>43</v>
@@ -3998,16 +4015,16 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>493</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M16" t="s">
         <v>36</v>
@@ -4039,7 +4056,7 @@
         <v>89</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>43</v>
@@ -4047,16 +4064,16 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>496</v>
-      </c>
       <c r="K17" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M17" t="s">
         <v>36</v>
@@ -4085,10 +4102,10 @@
         <v>90</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>497</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>498</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>43</v>
@@ -4096,16 +4113,16 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>500</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M18" t="s">
         <v>36</v>
@@ -4134,10 +4151,10 @@
         <v>91</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>502</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>43</v>
@@ -4145,16 +4162,16 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>505</v>
-      </c>
       <c r="L19" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M19" t="s">
         <v>36</v>
@@ -4186,7 +4203,7 @@
         <v>93</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>43</v>
@@ -4195,11 +4212,11 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="M20" t="s">
         <v>94</v>
@@ -4261,13 +4278,13 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="L21" s="2" t="s">
         <v>510</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>511</v>
       </c>
       <c r="M21" t="s">
         <v>94</v>
@@ -4317,10 +4334,10 @@
         <v>107</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>108</v>
@@ -4422,7 +4439,7 @@
         <v>120</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>43</v>
@@ -4431,11 +4448,11 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" s="2" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="K24" s="2"/>
       <c r="L24" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="M24" t="s">
         <v>94</v>
@@ -4485,7 +4502,7 @@
         <v>123</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>43</v>
@@ -4496,7 +4513,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="M25" t="s">
         <v>124</v>
@@ -4543,10 +4560,10 @@
         <v>130</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>518</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>519</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>43</v>
@@ -4555,13 +4572,13 @@
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="L26" s="2" t="s">
         <v>521</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>522</v>
       </c>
       <c r="M26" t="s">
         <v>36</v>
@@ -4587,10 +4604,10 @@
         <v>22</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>131</v>
@@ -4604,10 +4621,10 @@
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" t="s">
@@ -4655,13 +4672,13 @@
         <v>22</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>43</v>
@@ -4672,7 +4689,7 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="M28" t="s">
         <v>133</v>
@@ -4698,10 +4715,10 @@
         <v>22</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>139</v>
@@ -4715,10 +4732,10 @@
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="L29" s="3"/>
       <c r="M29" t="s">
@@ -4766,13 +4783,13 @@
         <v>22</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>43</v>
@@ -4783,7 +4800,7 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="M30" t="s">
         <v>141</v>
@@ -4809,13 +4826,13 @@
         <v>22</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>531</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>108</v>
@@ -4826,10 +4843,10 @@
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="L31" s="3"/>
       <c r="M31" t="s">
@@ -4877,13 +4894,13 @@
         <v>22</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>151</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>108</v>
@@ -4894,10 +4911,10 @@
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
       <c r="J32" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="K32" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="L32" s="3"/>
       <c r="M32" t="s">
@@ -4945,13 +4962,13 @@
         <v>22</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>43</v>
@@ -4962,7 +4979,7 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="M33" t="s">
         <v>152</v>
@@ -5006,13 +5023,13 @@
         <v>22</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>158</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>108</v>
@@ -5067,13 +5084,13 @@
         <v>22</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>23</v>
@@ -5111,13 +5128,13 @@
         <v>22</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>108</v>
@@ -5128,10 +5145,10 @@
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="J36" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>538</v>
       </c>
       <c r="L36" s="3"/>
       <c r="M36" t="s">
@@ -5176,13 +5193,13 @@
         <v>22</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>172</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>108</v>
@@ -5193,10 +5210,10 @@
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
       <c r="J37" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>538</v>
       </c>
       <c r="L37" s="3"/>
       <c r="M37" t="s">
@@ -5241,13 +5258,13 @@
         <v>22</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>177</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>108</v>
@@ -5258,10 +5275,10 @@
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="J38" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="L38" s="3"/>
       <c r="M38" t="s">
@@ -5288,13 +5305,13 @@
         <v>22</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>108</v>
@@ -5305,10 +5322,10 @@
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
       <c r="J39" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="K39" s="2" t="s">
         <v>543</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>544</v>
       </c>
       <c r="L39" s="3"/>
       <c r="M39" t="s">
@@ -5362,10 +5379,10 @@
         <v>187</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>545</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>546</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>43</v>
@@ -5376,7 +5393,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M40" t="s">
         <v>36</v>
@@ -5402,13 +5419,13 @@
         <v>22</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>108</v>
@@ -5445,13 +5462,13 @@
         <v>22</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>108</v>
@@ -5488,7 +5505,7 @@
         <v>22</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>190</v>
@@ -5543,10 +5560,10 @@
         <v>195</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>108</v>
@@ -5595,10 +5612,10 @@
         <v>200</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>108</v>
@@ -5647,10 +5664,10 @@
         <v>205</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>108</v>
@@ -5661,7 +5678,7 @@
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
       <c r="J46" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="K46" s="2"/>
       <c r="L46" s="3"/>
@@ -5692,7 +5709,7 @@
         <v>22</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>209</v>
@@ -5744,13 +5761,13 @@
         <v>22</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>108</v>
@@ -5799,10 +5816,10 @@
         <v>218</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>108</v>
@@ -5813,10 +5830,10 @@
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
       <c r="J49" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="K49" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="L49" s="3"/>
       <c r="M49" t="s">
@@ -5846,10 +5863,10 @@
         <v>220</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>43</v>
@@ -5859,10 +5876,10 @@
       <c r="I50" s="3"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="L50" s="2" t="s">
         <v>559</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>560</v>
       </c>
       <c r="M50" t="s">
         <v>36</v>
@@ -5891,10 +5908,10 @@
         <v>221</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>108</v>
@@ -5905,10 +5922,10 @@
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
       <c r="J51" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="K51" s="2" t="s">
         <v>562</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="L51" s="2"/>
       <c r="M51" t="s">
@@ -5938,10 +5955,10 @@
         <v>222</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>43</v>
@@ -5950,13 +5967,13 @@
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="K52" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>566</v>
-      </c>
       <c r="L52" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="M52" t="s">
         <v>223</v>
@@ -5997,7 +6014,7 @@
         <v>22</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>229</v>
@@ -6043,10 +6060,10 @@
         <v>231</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>108</v>
@@ -6057,10 +6074,10 @@
       <c r="H54" s="3"/>
       <c r="I54" s="3"/>
       <c r="J54" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="K54" s="2" t="s">
         <v>568</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>569</v>
       </c>
       <c r="L54" s="2"/>
       <c r="M54" t="s">
@@ -6102,10 +6119,10 @@
         <v>237</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>43</v>
@@ -6116,7 +6133,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="M55" t="s">
         <v>36</v>
@@ -6157,13 +6174,13 @@
       <c r="H56" s="3"/>
       <c r="I56" s="3"/>
       <c r="J56" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="K56" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="K56" s="2" t="s">
+      <c r="L56" s="2" t="s">
         <v>573</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>574</v>
       </c>
       <c r="M56" t="s">
         <v>240</v>
@@ -6223,10 +6240,10 @@
       <c r="I57" s="3"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="M57" t="s">
         <v>36</v>
@@ -6273,10 +6290,10 @@
         <v>248</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>108</v>
@@ -6287,10 +6304,10 @@
       <c r="H58" s="3"/>
       <c r="I58" s="3"/>
       <c r="J58" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L58" s="2"/>
       <c r="M58" t="s">
@@ -6396,11 +6413,11 @@
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
       <c r="J60" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="K60" s="2"/>
       <c r="L60" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="M60" t="s">
         <v>252</v>
@@ -6447,10 +6464,10 @@
         <v>263</v>
       </c>
       <c r="D61" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="E61" s="2" t="s">
         <v>580</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>581</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>43</v>
@@ -6460,10 +6477,10 @@
       <c r="I61" s="3"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="L61" s="2" t="s">
         <v>582</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>583</v>
       </c>
       <c r="M61" t="s">
         <v>264</v>
@@ -6507,7 +6524,7 @@
         <v>22</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>270</v>
@@ -6526,7 +6543,7 @@
       </c>
       <c r="K62" s="2"/>
       <c r="L62" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M62" t="s">
         <v>36</v>
@@ -6552,13 +6569,13 @@
         <v>22</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>43</v>
@@ -6569,7 +6586,7 @@
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
       <c r="L63" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M63" t="s">
         <v>272</v>
@@ -6616,13 +6633,13 @@
         <v>22</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>43</v>
@@ -6633,7 +6650,7 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
       <c r="L64" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M64" t="s">
         <v>36</v>
@@ -6659,13 +6676,13 @@
         <v>22</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="D65" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E65" s="2" t="s">
         <v>587</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>588</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>43</v>
@@ -6676,7 +6693,7 @@
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
       <c r="L65" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="M65" t="s">
         <v>280</v>
@@ -6726,7 +6743,7 @@
         <v>286</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>287</v>
@@ -6742,7 +6759,7 @@
       </c>
       <c r="K66" s="2"/>
       <c r="L66" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M66" t="s">
         <v>36</v>
@@ -6771,7 +6788,7 @@
         <v>288</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>289</v>
@@ -6787,7 +6804,7 @@
       </c>
       <c r="K67" s="2"/>
       <c r="L67" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M67" t="s">
         <v>36</v>
@@ -6813,13 +6830,13 @@
         <v>22</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>108</v>
@@ -6879,13 +6896,13 @@
         <v>22</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>296</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>43</v>
@@ -6896,7 +6913,7 @@
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
       <c r="L69" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="M69" t="s">
         <v>290</v>
@@ -6943,13 +6960,13 @@
         <v>22</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D70" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>595</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>596</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>43</v>
@@ -6959,10 +6976,10 @@
       <c r="I70" s="3"/>
       <c r="J70" s="2"/>
       <c r="K70" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="L70" s="2" t="s">
         <v>597</v>
-      </c>
-      <c r="L70" s="2" t="s">
-        <v>598</v>
       </c>
       <c r="M70" t="s">
         <v>36</v>
@@ -6991,7 +7008,7 @@
         <v>22</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>426</v>
@@ -7007,10 +7024,10 @@
       <c r="I71" s="3"/>
       <c r="J71" s="2"/>
       <c r="K71" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M71" t="s">
         <v>36</v>
@@ -7036,13 +7053,13 @@
         <v>22</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>428</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>43</v>
@@ -7051,13 +7068,13 @@
       <c r="H72" s="3"/>
       <c r="I72" s="3"/>
       <c r="J72" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M72" t="s">
         <v>36</v>
@@ -7083,13 +7100,13 @@
         <v>22</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>429</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>43</v>
@@ -7098,11 +7115,11 @@
       <c r="H73" s="3"/>
       <c r="I73" s="3"/>
       <c r="J73" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="K73" s="2"/>
       <c r="L73" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M73" t="s">
         <v>430</v>
@@ -7146,13 +7163,13 @@
         <v>22</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>436</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>43</v>
@@ -7161,13 +7178,13 @@
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
       <c r="J74" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="M74" t="s">
         <v>437</v>
@@ -7214,13 +7231,13 @@
         <v>22</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D75" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>606</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>607</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>108</v>
@@ -7229,7 +7246,7 @@
       <c r="H75" s="3"/>
       <c r="I75" s="3"/>
       <c r="J75" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="K75" s="2"/>
       <c r="L75" s="2"/>
@@ -7246,10 +7263,10 @@
         <v>445</v>
       </c>
       <c r="Z75" s="1" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="76" spans="1:26" ht="270" x14ac:dyDescent="0.25">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="76" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -7257,13 +7274,13 @@
         <v>22</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D76" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="E76" s="2" t="s">
         <v>609</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>610</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>43</v>
@@ -7289,7 +7306,7 @@
         <v>52</v>
       </c>
       <c r="Z76" s="1" t="s">
-        <v>447</v>
+        <v>749</v>
       </c>
     </row>
     <row r="77" spans="1:26" ht="390" x14ac:dyDescent="0.25">
@@ -7316,10 +7333,10 @@
       <c r="I77" s="3"/>
       <c r="J77" s="2"/>
       <c r="K77" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="L77" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="L77" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="M77" t="s">
         <v>301</v>
@@ -7369,10 +7386,10 @@
         <v>307</v>
       </c>
       <c r="D78" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>613</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>614</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>43</v>
@@ -7381,13 +7398,13 @@
       <c r="H78" s="3"/>
       <c r="I78" s="3"/>
       <c r="J78" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="K78" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="K78" s="2" t="s">
+      <c r="L78" s="2" t="s">
         <v>616</v>
-      </c>
-      <c r="L78" s="2" t="s">
-        <v>617</v>
       </c>
       <c r="M78" s="1" t="s">
         <v>308</v>
@@ -7437,10 +7454,10 @@
         <v>316</v>
       </c>
       <c r="D79" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="E79" s="3" t="s">
         <v>618</v>
-      </c>
-      <c r="E79" s="3" t="s">
-        <v>619</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>43</v>
@@ -7448,14 +7465,14 @@
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="J79" s="2" t="s">
         <v>620</v>
-      </c>
-      <c r="J79" s="2" t="s">
-        <v>621</v>
       </c>
       <c r="K79" s="2"/>
       <c r="L79" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M79" t="s">
         <v>317</v>
@@ -7505,10 +7522,10 @@
         <v>322</v>
       </c>
       <c r="D80" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="E80" s="3" t="s">
         <v>622</v>
-      </c>
-      <c r="E80" s="3" t="s">
-        <v>623</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>43</v>
@@ -7516,14 +7533,14 @@
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
       <c r="I80" s="3" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J80" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="K80" s="2"/>
       <c r="L80" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M80" t="s">
         <v>317</v>
@@ -7570,10 +7587,10 @@
         <v>325</v>
       </c>
       <c r="D81" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E81" s="3" t="s">
         <v>625</v>
-      </c>
-      <c r="E81" s="3" t="s">
-        <v>626</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>43</v>
@@ -7581,14 +7598,14 @@
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
       <c r="I81" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="K81" s="2"/>
       <c r="L81" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M81" t="s">
         <v>326</v>
@@ -7635,10 +7652,10 @@
         <v>329</v>
       </c>
       <c r="D82" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="E82" s="3" t="s">
         <v>628</v>
-      </c>
-      <c r="E82" s="3" t="s">
-        <v>629</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>43</v>
@@ -7646,14 +7663,14 @@
       <c r="G82" s="3"/>
       <c r="H82" s="3"/>
       <c r="I82" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="K82" s="2"/>
       <c r="L82" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M82" t="s">
         <v>330</v>
@@ -7697,13 +7714,13 @@
         <v>22</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D83" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="E83" s="3" t="s">
         <v>631</v>
-      </c>
-      <c r="E83" s="3" t="s">
-        <v>632</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>43</v>
@@ -7711,14 +7728,14 @@
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
       <c r="I83" s="3" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="J83" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="K83" s="2"/>
       <c r="L83" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M83" t="s">
         <v>36</v>
@@ -7762,13 +7779,13 @@
         <v>22</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D84" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="E84" s="3" t="s">
         <v>634</v>
-      </c>
-      <c r="E84" s="3" t="s">
-        <v>635</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>43</v>
@@ -7776,14 +7793,14 @@
       <c r="G84" s="3"/>
       <c r="H84" s="3"/>
       <c r="I84" s="3" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J84" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="K84" s="2"/>
       <c r="L84" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M84" t="s">
         <v>36</v>
@@ -7830,10 +7847,10 @@
         <v>333</v>
       </c>
       <c r="D85" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="E85" s="3" t="s">
         <v>637</v>
-      </c>
-      <c r="E85" s="3" t="s">
-        <v>638</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>43</v>
@@ -7841,16 +7858,16 @@
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
       <c r="I85" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="J85" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="J85" s="2" t="s">
+      <c r="K85" s="2" t="s">
         <v>640</v>
       </c>
-      <c r="K85" s="2" t="s">
-        <v>641</v>
-      </c>
       <c r="L85" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M85" t="s">
         <v>334</v>
@@ -7897,10 +7914,10 @@
         <v>337</v>
       </c>
       <c r="D86" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E86" s="5" t="s">
         <v>642</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>643</v>
       </c>
       <c r="F86" s="4" t="s">
         <v>43</v>
@@ -7908,14 +7925,14 @@
       <c r="G86" s="5"/>
       <c r="H86" s="5"/>
       <c r="I86" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="K86" s="4"/>
       <c r="L86" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M86" s="1" t="s">
         <v>338</v>
@@ -7948,7 +7965,7 @@
         <v>298</v>
       </c>
       <c r="Z86" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="87" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -7962,10 +7979,10 @@
         <v>339</v>
       </c>
       <c r="D87" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>43</v>
@@ -7974,11 +7991,11 @@
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
       <c r="J87" s="2" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K87" s="2"/>
       <c r="L87" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M87" s="1" t="s">
         <v>340</v>
@@ -8022,13 +8039,13 @@
         <v>22</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D88" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="E88" s="2" t="s">
         <v>648</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>649</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>43</v>
@@ -8036,16 +8053,16 @@
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
       <c r="I88" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="K88" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="J88" s="2" t="s">
-        <v>647</v>
-      </c>
-      <c r="K88" s="2" t="s">
-        <v>651</v>
-      </c>
       <c r="L88" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M88" t="s">
         <v>346</v>
@@ -8108,10 +8125,10 @@
       <c r="I89" s="3"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="L89" s="2" t="s">
         <v>652</v>
-      </c>
-      <c r="L89" s="2" t="s">
-        <v>653</v>
       </c>
       <c r="M89" t="s">
         <v>346</v>
@@ -8164,7 +8181,7 @@
         <v>354</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>43</v>
@@ -8173,13 +8190,13 @@
       <c r="H90" s="3"/>
       <c r="I90" s="3"/>
       <c r="J90" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="K90" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="K90" s="2" t="s">
-        <v>656</v>
-      </c>
       <c r="L90" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M90" t="s">
         <v>355</v>
@@ -8229,7 +8246,7 @@
         <v>359</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>43</v>
@@ -8238,11 +8255,11 @@
       <c r="H91" s="3"/>
       <c r="I91" s="3"/>
       <c r="J91" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K91" s="2"/>
       <c r="L91" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M91" t="s">
         <v>355</v>
@@ -8292,7 +8309,7 @@
         <v>362</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>43</v>
@@ -8301,11 +8318,11 @@
       <c r="H92" s="3"/>
       <c r="I92" s="3"/>
       <c r="J92" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K92" s="2"/>
       <c r="L92" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M92" t="s">
         <v>355</v>
@@ -8355,7 +8372,7 @@
         <v>364</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>43</v>
@@ -8364,11 +8381,11 @@
       <c r="H93" s="3"/>
       <c r="I93" s="3"/>
       <c r="J93" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K93" s="2"/>
       <c r="L93" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M93" t="s">
         <v>355</v>
@@ -8415,10 +8432,10 @@
         <v>365</v>
       </c>
       <c r="D94" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="E94" s="2" t="s">
         <v>661</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>662</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>43</v>
@@ -8427,11 +8444,11 @@
       <c r="H94" s="3"/>
       <c r="I94" s="3"/>
       <c r="J94" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K94" s="2"/>
       <c r="L94" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M94" t="s">
         <v>355</v>
@@ -8481,7 +8498,7 @@
         <v>367</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>43</v>
@@ -8490,11 +8507,11 @@
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
       <c r="J95" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K95" s="2"/>
       <c r="L95" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M95" t="s">
         <v>355</v>
@@ -8541,10 +8558,10 @@
         <v>368</v>
       </c>
       <c r="D96" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="E96" s="2" t="s">
         <v>664</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>665</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>43</v>
@@ -8553,11 +8570,11 @@
       <c r="H96" s="3"/>
       <c r="I96" s="3"/>
       <c r="J96" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K96" s="2"/>
       <c r="L96" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M96" t="s">
         <v>355</v>
@@ -8607,7 +8624,7 @@
         <v>370</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>43</v>
@@ -8616,11 +8633,11 @@
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
       <c r="J97" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K97" s="2"/>
       <c r="L97" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M97" t="s">
         <v>355</v>
@@ -8670,7 +8687,7 @@
         <v>372</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>43</v>
@@ -8679,11 +8696,11 @@
       <c r="H98" s="3"/>
       <c r="I98" s="3"/>
       <c r="J98" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K98" s="2"/>
       <c r="L98" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M98" t="s">
         <v>355</v>
@@ -8733,7 +8750,7 @@
         <v>374</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>43</v>
@@ -8742,11 +8759,11 @@
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
       <c r="J99" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K99" s="2"/>
       <c r="L99" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M99" t="s">
         <v>355</v>
@@ -8796,7 +8813,7 @@
         <v>376</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>43</v>
@@ -8805,11 +8822,11 @@
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
       <c r="J100" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K100" s="2"/>
       <c r="L100" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M100" t="s">
         <v>355</v>
@@ -8859,7 +8876,7 @@
         <v>378</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>43</v>
@@ -8868,11 +8885,11 @@
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
       <c r="J101" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K101" s="2"/>
       <c r="L101" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M101" t="s">
         <v>355</v>
@@ -8922,7 +8939,7 @@
         <v>380</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>43</v>
@@ -8931,11 +8948,11 @@
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
       <c r="J102" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K102" s="2"/>
       <c r="L102" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M102" t="s">
         <v>355</v>
@@ -8985,7 +9002,7 @@
         <v>382</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>43</v>
@@ -8994,11 +9011,11 @@
       <c r="H103" s="3"/>
       <c r="I103" s="3"/>
       <c r="J103" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K103" s="2"/>
       <c r="L103" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M103" t="s">
         <v>355</v>
@@ -9048,7 +9065,7 @@
         <v>384</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>43</v>
@@ -9057,11 +9074,11 @@
       <c r="H104" s="3"/>
       <c r="I104" s="3"/>
       <c r="J104" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K104" s="2"/>
       <c r="L104" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M104" t="s">
         <v>355</v>
@@ -9111,7 +9128,7 @@
         <v>386</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>43</v>
@@ -9120,11 +9137,11 @@
       <c r="H105" s="3"/>
       <c r="I105" s="3"/>
       <c r="J105" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K105" s="2"/>
       <c r="L105" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M105" t="s">
         <v>355</v>
@@ -9174,7 +9191,7 @@
         <v>388</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>43</v>
@@ -9183,11 +9200,11 @@
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
       <c r="J106" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K106" s="2"/>
       <c r="L106" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M106" t="s">
         <v>355</v>
@@ -9237,7 +9254,7 @@
         <v>390</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>43</v>
@@ -9246,11 +9263,11 @@
       <c r="H107" s="3"/>
       <c r="I107" s="3"/>
       <c r="J107" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K107" s="2"/>
       <c r="L107" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M107" t="s">
         <v>355</v>
@@ -9300,7 +9317,7 @@
         <v>392</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>43</v>
@@ -9309,11 +9326,11 @@
       <c r="H108" s="3"/>
       <c r="I108" s="3"/>
       <c r="J108" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K108" s="2"/>
       <c r="L108" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M108" t="s">
         <v>355</v>
@@ -9363,7 +9380,7 @@
         <v>394</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>43</v>
@@ -9372,11 +9389,11 @@
       <c r="H109" s="3"/>
       <c r="I109" s="3"/>
       <c r="J109" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K109" s="2"/>
       <c r="L109" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M109" t="s">
         <v>355</v>
@@ -9420,13 +9437,13 @@
         <v>22</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D110" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="E110" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>680</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>43</v>
@@ -9435,11 +9452,11 @@
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
       <c r="J110" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="K110" s="2"/>
       <c r="L110" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M110" t="s">
         <v>395</v>
@@ -9489,7 +9506,7 @@
         <v>399</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>43</v>
@@ -9498,11 +9515,11 @@
       <c r="H111" s="3"/>
       <c r="I111" s="3"/>
       <c r="J111" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="K111" s="2"/>
       <c r="L111" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M111" t="s">
         <v>400</v>
@@ -9549,10 +9566,10 @@
         <v>404</v>
       </c>
       <c r="D112" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="E112" s="2" t="s">
         <v>684</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>685</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>43</v>
@@ -9561,11 +9578,11 @@
       <c r="H112" s="3"/>
       <c r="I112" s="3"/>
       <c r="J112" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="K112" s="2"/>
       <c r="L112" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M112" t="s">
         <v>405</v>
@@ -9609,13 +9626,13 @@
         <v>22</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>43</v>
@@ -9624,11 +9641,11 @@
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
       <c r="J113" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="K113" s="2"/>
       <c r="L113" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M113" s="1" t="s">
         <v>409</v>
@@ -9675,7 +9692,7 @@
         <v>22</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="D114" s="2" t="s">
         <v>416</v>
@@ -9690,11 +9707,11 @@
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
       <c r="J114" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="K114" s="2"/>
       <c r="L114" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M114" s="1" t="s">
         <v>409</v>
@@ -9741,7 +9758,7 @@
         <v>22</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D115" s="2" t="s">
         <v>418</v>
@@ -9756,11 +9773,11 @@
       <c r="H115" s="3"/>
       <c r="I115" s="3"/>
       <c r="J115" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="K115" s="2"/>
       <c r="L115" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="M115" s="1" t="s">
         <v>409</v>
@@ -9807,13 +9824,13 @@
         <v>22</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>43</v>
@@ -9822,7 +9839,7 @@
       <c r="H116" s="3"/>
       <c r="I116" s="3"/>
       <c r="J116" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="K116" s="2"/>
       <c r="L116" s="2"/>
@@ -9850,13 +9867,13 @@
         <v>22</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>43</v>
@@ -9865,7 +9882,7 @@
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
       <c r="J117" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K117" s="2"/>
       <c r="L117" s="2"/>
@@ -9893,13 +9910,13 @@
         <v>22</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>43</v>
@@ -9908,7 +9925,7 @@
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
       <c r="J118" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="K118" s="2"/>
       <c r="L118" s="2"/>
@@ -9936,13 +9953,13 @@
         <v>22</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>43</v>
@@ -9951,7 +9968,7 @@
       <c r="H119" s="3"/>
       <c r="I119" s="3"/>
       <c r="J119" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="K119" s="2"/>
       <c r="L119" s="2"/>
@@ -9979,13 +9996,13 @@
         <v>22</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F120" s="2" t="s">
         <v>43</v>
@@ -9994,7 +10011,7 @@
       <c r="H120" s="3"/>
       <c r="I120" s="3"/>
       <c r="J120" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="K120" s="2"/>
       <c r="L120" s="2"/>
@@ -10022,13 +10039,13 @@
         <v>22</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>43</v>
@@ -10037,7 +10054,7 @@
       <c r="H121" s="3"/>
       <c r="I121" s="3"/>
       <c r="J121" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K121" s="2"/>
       <c r="L121" s="2"/>
@@ -10083,13 +10100,13 @@
         <v>22</v>
       </c>
       <c r="C122" s="6" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>43</v>
@@ -10098,7 +10115,7 @@
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
       <c r="J122" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K122" s="2"/>
       <c r="L122" s="2"/>
@@ -10119,6 +10136,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Z1" xr:uid="{5DD590CF-60F3-474A-8CF6-CAFB2AFA3E98}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correct sf36 n items
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-FRA.xlsx
+++ b/baseline/data_processing_elements-FRA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\FRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CF1CCA-1863-4B33-A3BC-34CA21583BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8FA2F2-0CDC-4190-908B-16CDF1F89BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CCDECE63-0FFC-4822-923F-34FACAF497E3}"/>
   </bookViews>
@@ -2771,7 +2771,7 @@
 temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
 select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
 temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE)) == 0,NA,
+na.rm = TRUE) == 0,NA,
 rowSums(mutate(.,
 temp_dis_vigorous1 = as.numeric(!is.na(dis_vigorous1)), 
 temp_dis_moderate1 = as.numeric(!is.na(dis_moderate1)),
@@ -2785,7 +2785,7 @@
 temp_dis_bath1 = as.numeric(!is.na(dis_bath1))) %&gt;%
 select(temp_dis_vigorous1, temp_dis_moderate1, temp_dis_lift1, temp_dis_climbseveral1, temp_dis_climbone1,
 temp_dis_bending1, temp_dis_walk2km_1, temp_dis_walk1km_1, temp_dis_walk100m_1, temp_dis_bath1), 
-na.rm = TRUE)))</t>
+na.rm = TRUE))</t>
   </si>
 </sst>
 </file>

</xml_diff>